<commit_message>
Swap household splitter for PLZ splitter, lock age and education
Per Ole:
- Alter is now fixed studywide at "20-29 Jahre" (drop the per-role age
  ranges since the LLM picks within the range itself at T=0.7)
- Ausbildung locked to "Bachelor" only (Master out)
- Postleitzahl is the new second splitter: "9000, 9403" (St. Gallen
  urban vs. Goldach more rural -> mild urban/rural signal)
- Haushalt back to a single fixed value "2 Personen 1 Kind" so we land
  exactly on 24 personas again

Math: 6 roles x 2 genders x 1 age x 1 household x 1 edu x 1 work-exp
x 2 PLZ = 24.

Also regenerates personas_24.xlsx via the updated generator script.
localStorage role_vars key v24 -> v25.

https://claude.ai/code/session_01TEFCvyf4eB4epJ3yuxH4cG
</commit_message>
<xml_diff>
--- a/personas_24.xlsx
+++ b/personas_24.xlsx
@@ -454,16 +454,16 @@
         <v>Männlich</v>
       </c>
       <c r="D2" t="str">
-        <v>23-26 Jahre</v>
+        <v>20-29 Jahre</v>
       </c>
       <c r="E2" t="str">
         <v>Schweiz</v>
       </c>
       <c r="F2" t="str">
-        <v>1 Person kein Kind</v>
+        <v>2 Personen 1 Kind</v>
       </c>
       <c r="G2" t="str">
-        <v>Bachelor / Master</v>
+        <v>Bachelor</v>
       </c>
       <c r="H2" t="str">
         <v>5-7 Jahre</v>
@@ -486,7 +486,7 @@
         <v>Männlich</v>
       </c>
       <c r="D3" t="str">
-        <v>23-26 Jahre</v>
+        <v>20-29 Jahre</v>
       </c>
       <c r="E3" t="str">
         <v>Schweiz</v>
@@ -495,7 +495,7 @@
         <v>2 Personen 1 Kind</v>
       </c>
       <c r="G3" t="str">
-        <v>Bachelor / Master</v>
+        <v>Bachelor</v>
       </c>
       <c r="H3" t="str">
         <v>5-7 Jahre</v>
@@ -504,7 +504,7 @@
         <v>Schweiz</v>
       </c>
       <c r="J3" t="str">
-        <v>9000</v>
+        <v>9403</v>
       </c>
     </row>
     <row r="4">
@@ -518,16 +518,16 @@
         <v>Weiblich</v>
       </c>
       <c r="D4" t="str">
-        <v>23-26 Jahre</v>
+        <v>20-29 Jahre</v>
       </c>
       <c r="E4" t="str">
         <v>Schweiz</v>
       </c>
       <c r="F4" t="str">
-        <v>1 Person kein Kind</v>
+        <v>2 Personen 1 Kind</v>
       </c>
       <c r="G4" t="str">
-        <v>Bachelor / Master</v>
+        <v>Bachelor</v>
       </c>
       <c r="H4" t="str">
         <v>5-7 Jahre</v>
@@ -550,7 +550,7 @@
         <v>Weiblich</v>
       </c>
       <c r="D5" t="str">
-        <v>23-26 Jahre</v>
+        <v>20-29 Jahre</v>
       </c>
       <c r="E5" t="str">
         <v>Schweiz</v>
@@ -559,7 +559,7 @@
         <v>2 Personen 1 Kind</v>
       </c>
       <c r="G5" t="str">
-        <v>Bachelor / Master</v>
+        <v>Bachelor</v>
       </c>
       <c r="H5" t="str">
         <v>5-7 Jahre</v>
@@ -568,7 +568,7 @@
         <v>Schweiz</v>
       </c>
       <c r="J5" t="str">
-        <v>9000</v>
+        <v>9403</v>
       </c>
     </row>
     <row r="6">
@@ -582,16 +582,16 @@
         <v>Männlich</v>
       </c>
       <c r="D6" t="str">
-        <v>25-31 Jahre</v>
+        <v>20-29 Jahre</v>
       </c>
       <c r="E6" t="str">
         <v>Schweiz</v>
       </c>
       <c r="F6" t="str">
-        <v>1 Person kein Kind</v>
+        <v>2 Personen 1 Kind</v>
       </c>
       <c r="G6" t="str">
-        <v>Bachelor / Master</v>
+        <v>Bachelor</v>
       </c>
       <c r="H6" t="str">
         <v>2-5 Jahre</v>
@@ -614,7 +614,7 @@
         <v>Männlich</v>
       </c>
       <c r="D7" t="str">
-        <v>25-31 Jahre</v>
+        <v>20-29 Jahre</v>
       </c>
       <c r="E7" t="str">
         <v>Schweiz</v>
@@ -623,7 +623,7 @@
         <v>2 Personen 1 Kind</v>
       </c>
       <c r="G7" t="str">
-        <v>Bachelor / Master</v>
+        <v>Bachelor</v>
       </c>
       <c r="H7" t="str">
         <v>2-5 Jahre</v>
@@ -632,7 +632,7 @@
         <v>Schweiz</v>
       </c>
       <c r="J7" t="str">
-        <v>9000</v>
+        <v>9403</v>
       </c>
     </row>
     <row r="8">
@@ -646,16 +646,16 @@
         <v>Weiblich</v>
       </c>
       <c r="D8" t="str">
-        <v>25-31 Jahre</v>
+        <v>20-29 Jahre</v>
       </c>
       <c r="E8" t="str">
         <v>Schweiz</v>
       </c>
       <c r="F8" t="str">
-        <v>1 Person kein Kind</v>
+        <v>2 Personen 1 Kind</v>
       </c>
       <c r="G8" t="str">
-        <v>Bachelor / Master</v>
+        <v>Bachelor</v>
       </c>
       <c r="H8" t="str">
         <v>2-5 Jahre</v>
@@ -678,7 +678,7 @@
         <v>Weiblich</v>
       </c>
       <c r="D9" t="str">
-        <v>25-31 Jahre</v>
+        <v>20-29 Jahre</v>
       </c>
       <c r="E9" t="str">
         <v>Schweiz</v>
@@ -687,7 +687,7 @@
         <v>2 Personen 1 Kind</v>
       </c>
       <c r="G9" t="str">
-        <v>Bachelor / Master</v>
+        <v>Bachelor</v>
       </c>
       <c r="H9" t="str">
         <v>2-5 Jahre</v>
@@ -696,7 +696,7 @@
         <v>Schweiz</v>
       </c>
       <c r="J9" t="str">
-        <v>9000</v>
+        <v>9403</v>
       </c>
     </row>
     <row r="10">
@@ -710,16 +710,16 @@
         <v>Männlich</v>
       </c>
       <c r="D10" t="str">
-        <v>22-28 Jahre</v>
+        <v>20-29 Jahre</v>
       </c>
       <c r="E10" t="str">
         <v>Schweiz</v>
       </c>
       <c r="F10" t="str">
-        <v>1 Person kein Kind</v>
+        <v>2 Personen 1 Kind</v>
       </c>
       <c r="G10" t="str">
-        <v>Bachelor / Master</v>
+        <v>Bachelor</v>
       </c>
       <c r="H10" t="str">
         <v>2-4 Jahre</v>
@@ -742,7 +742,7 @@
         <v>Männlich</v>
       </c>
       <c r="D11" t="str">
-        <v>22-28 Jahre</v>
+        <v>20-29 Jahre</v>
       </c>
       <c r="E11" t="str">
         <v>Schweiz</v>
@@ -751,7 +751,7 @@
         <v>2 Personen 1 Kind</v>
       </c>
       <c r="G11" t="str">
-        <v>Bachelor / Master</v>
+        <v>Bachelor</v>
       </c>
       <c r="H11" t="str">
         <v>2-4 Jahre</v>
@@ -760,7 +760,7 @@
         <v>Schweiz</v>
       </c>
       <c r="J11" t="str">
-        <v>9000</v>
+        <v>9403</v>
       </c>
     </row>
     <row r="12">
@@ -774,16 +774,16 @@
         <v>Weiblich</v>
       </c>
       <c r="D12" t="str">
-        <v>22-28 Jahre</v>
+        <v>20-29 Jahre</v>
       </c>
       <c r="E12" t="str">
         <v>Schweiz</v>
       </c>
       <c r="F12" t="str">
-        <v>1 Person kein Kind</v>
+        <v>2 Personen 1 Kind</v>
       </c>
       <c r="G12" t="str">
-        <v>Bachelor / Master</v>
+        <v>Bachelor</v>
       </c>
       <c r="H12" t="str">
         <v>2-4 Jahre</v>
@@ -806,7 +806,7 @@
         <v>Weiblich</v>
       </c>
       <c r="D13" t="str">
-        <v>22-28 Jahre</v>
+        <v>20-29 Jahre</v>
       </c>
       <c r="E13" t="str">
         <v>Schweiz</v>
@@ -815,7 +815,7 @@
         <v>2 Personen 1 Kind</v>
       </c>
       <c r="G13" t="str">
-        <v>Bachelor / Master</v>
+        <v>Bachelor</v>
       </c>
       <c r="H13" t="str">
         <v>2-4 Jahre</v>
@@ -824,7 +824,7 @@
         <v>Schweiz</v>
       </c>
       <c r="J13" t="str">
-        <v>9000</v>
+        <v>9403</v>
       </c>
     </row>
     <row r="14">
@@ -838,16 +838,16 @@
         <v>Männlich</v>
       </c>
       <c r="D14" t="str">
-        <v>26-30 Jahre</v>
+        <v>20-29 Jahre</v>
       </c>
       <c r="E14" t="str">
         <v>Schweiz</v>
       </c>
       <c r="F14" t="str">
-        <v>1 Person kein Kind</v>
+        <v>2 Personen 1 Kind</v>
       </c>
       <c r="G14" t="str">
-        <v>Bachelor / Master</v>
+        <v>Bachelor</v>
       </c>
       <c r="H14" t="str">
         <v>2-4 Jahre</v>
@@ -870,7 +870,7 @@
         <v>Männlich</v>
       </c>
       <c r="D15" t="str">
-        <v>26-30 Jahre</v>
+        <v>20-29 Jahre</v>
       </c>
       <c r="E15" t="str">
         <v>Schweiz</v>
@@ -879,7 +879,7 @@
         <v>2 Personen 1 Kind</v>
       </c>
       <c r="G15" t="str">
-        <v>Bachelor / Master</v>
+        <v>Bachelor</v>
       </c>
       <c r="H15" t="str">
         <v>2-4 Jahre</v>
@@ -888,7 +888,7 @@
         <v>Schweiz</v>
       </c>
       <c r="J15" t="str">
-        <v>9000</v>
+        <v>9403</v>
       </c>
     </row>
     <row r="16">
@@ -902,16 +902,16 @@
         <v>Weiblich</v>
       </c>
       <c r="D16" t="str">
-        <v>26-30 Jahre</v>
+        <v>20-29 Jahre</v>
       </c>
       <c r="E16" t="str">
         <v>Schweiz</v>
       </c>
       <c r="F16" t="str">
-        <v>1 Person kein Kind</v>
+        <v>2 Personen 1 Kind</v>
       </c>
       <c r="G16" t="str">
-        <v>Bachelor / Master</v>
+        <v>Bachelor</v>
       </c>
       <c r="H16" t="str">
         <v>2-4 Jahre</v>
@@ -934,7 +934,7 @@
         <v>Weiblich</v>
       </c>
       <c r="D17" t="str">
-        <v>26-30 Jahre</v>
+        <v>20-29 Jahre</v>
       </c>
       <c r="E17" t="str">
         <v>Schweiz</v>
@@ -943,7 +943,7 @@
         <v>2 Personen 1 Kind</v>
       </c>
       <c r="G17" t="str">
-        <v>Bachelor / Master</v>
+        <v>Bachelor</v>
       </c>
       <c r="H17" t="str">
         <v>2-4 Jahre</v>
@@ -952,7 +952,7 @@
         <v>Schweiz</v>
       </c>
       <c r="J17" t="str">
-        <v>9000</v>
+        <v>9403</v>
       </c>
     </row>
     <row r="18">
@@ -966,16 +966,16 @@
         <v>Männlich</v>
       </c>
       <c r="D18" t="str">
-        <v>22-25 Jahre</v>
+        <v>20-29 Jahre</v>
       </c>
       <c r="E18" t="str">
         <v>Schweiz</v>
       </c>
       <c r="F18" t="str">
-        <v>1 Person kein Kind</v>
+        <v>2 Personen 1 Kind</v>
       </c>
       <c r="G18" t="str">
-        <v>Bachelor / Master</v>
+        <v>Bachelor</v>
       </c>
       <c r="H18" t="str">
         <v>4-6 Jahre</v>
@@ -998,7 +998,7 @@
         <v>Männlich</v>
       </c>
       <c r="D19" t="str">
-        <v>22-25 Jahre</v>
+        <v>20-29 Jahre</v>
       </c>
       <c r="E19" t="str">
         <v>Schweiz</v>
@@ -1007,7 +1007,7 @@
         <v>2 Personen 1 Kind</v>
       </c>
       <c r="G19" t="str">
-        <v>Bachelor / Master</v>
+        <v>Bachelor</v>
       </c>
       <c r="H19" t="str">
         <v>4-6 Jahre</v>
@@ -1016,7 +1016,7 @@
         <v>Schweiz</v>
       </c>
       <c r="J19" t="str">
-        <v>9000</v>
+        <v>9403</v>
       </c>
     </row>
     <row r="20">
@@ -1030,16 +1030,16 @@
         <v>Weiblich</v>
       </c>
       <c r="D20" t="str">
-        <v>22-25 Jahre</v>
+        <v>20-29 Jahre</v>
       </c>
       <c r="E20" t="str">
         <v>Schweiz</v>
       </c>
       <c r="F20" t="str">
-        <v>1 Person kein Kind</v>
+        <v>2 Personen 1 Kind</v>
       </c>
       <c r="G20" t="str">
-        <v>Bachelor / Master</v>
+        <v>Bachelor</v>
       </c>
       <c r="H20" t="str">
         <v>4-6 Jahre</v>
@@ -1062,7 +1062,7 @@
         <v>Weiblich</v>
       </c>
       <c r="D21" t="str">
-        <v>22-25 Jahre</v>
+        <v>20-29 Jahre</v>
       </c>
       <c r="E21" t="str">
         <v>Schweiz</v>
@@ -1071,7 +1071,7 @@
         <v>2 Personen 1 Kind</v>
       </c>
       <c r="G21" t="str">
-        <v>Bachelor / Master</v>
+        <v>Bachelor</v>
       </c>
       <c r="H21" t="str">
         <v>4-6 Jahre</v>
@@ -1080,7 +1080,7 @@
         <v>Schweiz</v>
       </c>
       <c r="J21" t="str">
-        <v>9000</v>
+        <v>9403</v>
       </c>
     </row>
     <row r="22">
@@ -1094,16 +1094,16 @@
         <v>Männlich</v>
       </c>
       <c r="D22" t="str">
-        <v>24-28 Jahre</v>
+        <v>20-29 Jahre</v>
       </c>
       <c r="E22" t="str">
         <v>Schweiz</v>
       </c>
       <c r="F22" t="str">
-        <v>1 Person kein Kind</v>
+        <v>2 Personen 1 Kind</v>
       </c>
       <c r="G22" t="str">
-        <v>Bachelor / Master</v>
+        <v>Bachelor</v>
       </c>
       <c r="H22" t="str">
         <v>5-7 Jahre</v>
@@ -1126,7 +1126,7 @@
         <v>Männlich</v>
       </c>
       <c r="D23" t="str">
-        <v>24-28 Jahre</v>
+        <v>20-29 Jahre</v>
       </c>
       <c r="E23" t="str">
         <v>Schweiz</v>
@@ -1135,7 +1135,7 @@
         <v>2 Personen 1 Kind</v>
       </c>
       <c r="G23" t="str">
-        <v>Bachelor / Master</v>
+        <v>Bachelor</v>
       </c>
       <c r="H23" t="str">
         <v>5-7 Jahre</v>
@@ -1144,7 +1144,7 @@
         <v>Schweiz</v>
       </c>
       <c r="J23" t="str">
-        <v>9000</v>
+        <v>9403</v>
       </c>
     </row>
     <row r="24">
@@ -1158,16 +1158,16 @@
         <v>Weiblich</v>
       </c>
       <c r="D24" t="str">
-        <v>24-28 Jahre</v>
+        <v>20-29 Jahre</v>
       </c>
       <c r="E24" t="str">
         <v>Schweiz</v>
       </c>
       <c r="F24" t="str">
-        <v>1 Person kein Kind</v>
+        <v>2 Personen 1 Kind</v>
       </c>
       <c r="G24" t="str">
-        <v>Bachelor / Master</v>
+        <v>Bachelor</v>
       </c>
       <c r="H24" t="str">
         <v>5-7 Jahre</v>
@@ -1190,7 +1190,7 @@
         <v>Weiblich</v>
       </c>
       <c r="D25" t="str">
-        <v>24-28 Jahre</v>
+        <v>20-29 Jahre</v>
       </c>
       <c r="E25" t="str">
         <v>Schweiz</v>
@@ -1199,7 +1199,7 @@
         <v>2 Personen 1 Kind</v>
       </c>
       <c r="G25" t="str">
-        <v>Bachelor / Master</v>
+        <v>Bachelor</v>
       </c>
       <c r="H25" t="str">
         <v>5-7 Jahre</v>
@@ -1208,7 +1208,7 @@
         <v>Schweiz</v>
       </c>
       <c r="J25" t="str">
-        <v>9000</v>
+        <v>9403</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add Jobbezeichnung/Jobbeschreibung/Avatar/Praeferenzen, drop Berufserfahrung
Renames Rolle to Jobbezeichnung mit ausgeschriebenen Titeln und ergaenzt pro
Rolle eine Jobbeschreibung (max. 3 Saetze), Avatar Eigenschaften und
Praeferenzen. Berufserfahrung-Spalte entfaellt.
</commit_message>
<xml_diff>
--- a/personas_24.xlsx
+++ b/personas_24.xlsx
@@ -397,18 +397,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J25"/>
+  <dimension ref="A1:L25"/>
   <cols>
     <col min="1" max="1" width="4.83203125" customWidth="1"/>
-    <col min="2" max="2" width="36.83203125" customWidth="1"/>
-    <col min="3" max="3" width="11.83203125" customWidth="1"/>
-    <col min="4" max="4" width="13.83203125" customWidth="1"/>
-    <col min="5" max="5" width="13.83203125" customWidth="1"/>
-    <col min="6" max="6" width="22.83203125" customWidth="1"/>
-    <col min="7" max="7" width="18.83203125" customWidth="1"/>
-    <col min="8" max="8" width="14.83203125" customWidth="1"/>
-    <col min="9" max="9" width="13.83203125" customWidth="1"/>
-    <col min="10" max="10" width="11.83203125" customWidth="1"/>
+    <col min="2" max="2" width="30.83203125" customWidth="1"/>
+    <col min="3" max="3" width="90.83203125" customWidth="1"/>
+    <col min="4" max="4" width="60.83203125" customWidth="1"/>
+    <col min="5" max="5" width="60.83203125" customWidth="1"/>
+    <col min="6" max="6" width="11.83203125" customWidth="1"/>
+    <col min="7" max="7" width="13.83203125" customWidth="1"/>
+    <col min="8" max="8" width="13.83203125" customWidth="1"/>
+    <col min="9" max="9" width="22.83203125" customWidth="1"/>
+    <col min="10" max="10" width="18.83203125" customWidth="1"/>
+    <col min="11" max="11" width="13.83203125" customWidth="1"/>
+    <col min="12" max="12" width="11.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -416,30 +418,36 @@
         <v>ID</v>
       </c>
       <c r="B1" t="str">
-        <v>Rolle</v>
+        <v>Jobbezeichnung</v>
       </c>
       <c r="C1" t="str">
+        <v>Jobbeschreibung</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Avatar Eigenschaften</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Präferenzen</v>
+      </c>
+      <c r="F1" t="str">
         <v>Geschlecht</v>
       </c>
-      <c r="D1" t="str">
+      <c r="G1" t="str">
         <v>Alter</v>
       </c>
-      <c r="E1" t="str">
+      <c r="H1" t="str">
         <v>Nationalitaet</v>
       </c>
-      <c r="F1" t="str">
+      <c r="I1" t="str">
         <v>Haushalt</v>
       </c>
-      <c r="G1" t="str">
+      <c r="J1" t="str">
         <v>Ausbildung</v>
       </c>
-      <c r="H1" t="str">
-        <v>Berufserfahrung</v>
-      </c>
-      <c r="I1" t="str">
+      <c r="K1" t="str">
         <v>Wohnsitzland</v>
       </c>
-      <c r="J1" t="str">
+      <c r="L1" t="str">
         <v>Postleitzahl</v>
       </c>
     </row>
@@ -448,30 +456,36 @@
         <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v>CEM (Customer Experience Manager)</v>
+        <v>Customer Experience Manager</v>
       </c>
       <c r="C2" t="str">
+        <v>Verantwortet die End-to-End-Customer-Journey und sorgt für konsistente, positive Kundenerlebnisse über alle Touchpoints. Analysiert Feedback, NPS und Verhaltensdaten, um Reibungspunkte zu reduzieren und Kundenbindung zu stärken. Arbeitet eng mit Marketing, Vertrieb und Service zusammen, um Prozesse kundenzentriert zu gestalten.</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Empathisch, datenaffin, prozessorientiert, kommunikativ, lösungsorientiert.</v>
+      </c>
+      <c r="E2" t="str">
+        <v>CRM-Tools (Salesforce, HubSpot), Customer-Journey-Mapping, NPS- und VoC-Programme, Cross-Functional Workshops.</v>
+      </c>
+      <c r="F2" t="str">
         <v>Männlich</v>
       </c>
-      <c r="D2" t="str">
-        <v>20-29 Jahre</v>
-      </c>
-      <c r="E2" t="str">
-        <v>Schweiz</v>
-      </c>
-      <c r="F2" t="str">
+      <c r="G2" t="str">
+        <v>20-29 Jahre</v>
+      </c>
+      <c r="H2" t="str">
+        <v>Schweiz</v>
+      </c>
+      <c r="I2" t="str">
         <v>1 Person kein Kind</v>
       </c>
-      <c r="G2" t="str">
-        <v>Bachelor</v>
-      </c>
-      <c r="H2" t="str">
-        <v>5-7 Jahre</v>
-      </c>
-      <c r="I2" t="str">
-        <v>Schweiz</v>
-      </c>
       <c r="J2" t="str">
+        <v>Bachelor</v>
+      </c>
+      <c r="K2" t="str">
+        <v>Schweiz</v>
+      </c>
+      <c r="L2" t="str">
         <v>9000</v>
       </c>
     </row>
@@ -480,30 +494,36 @@
         <v>2</v>
       </c>
       <c r="B3" t="str">
-        <v>CEM (Customer Experience Manager)</v>
+        <v>Customer Experience Manager</v>
       </c>
       <c r="C3" t="str">
+        <v>Verantwortet die End-to-End-Customer-Journey und sorgt für konsistente, positive Kundenerlebnisse über alle Touchpoints. Analysiert Feedback, NPS und Verhaltensdaten, um Reibungspunkte zu reduzieren und Kundenbindung zu stärken. Arbeitet eng mit Marketing, Vertrieb und Service zusammen, um Prozesse kundenzentriert zu gestalten.</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Empathisch, datenaffin, prozessorientiert, kommunikativ, lösungsorientiert.</v>
+      </c>
+      <c r="E3" t="str">
+        <v>CRM-Tools (Salesforce, HubSpot), Customer-Journey-Mapping, NPS- und VoC-Programme, Cross-Functional Workshops.</v>
+      </c>
+      <c r="F3" t="str">
         <v>Männlich</v>
       </c>
-      <c r="D3" t="str">
-        <v>20-29 Jahre</v>
-      </c>
-      <c r="E3" t="str">
-        <v>Schweiz</v>
-      </c>
-      <c r="F3" t="str">
+      <c r="G3" t="str">
+        <v>20-29 Jahre</v>
+      </c>
+      <c r="H3" t="str">
+        <v>Schweiz</v>
+      </c>
+      <c r="I3" t="str">
         <v>2 Personen 1 Kind</v>
       </c>
-      <c r="G3" t="str">
-        <v>Bachelor</v>
-      </c>
-      <c r="H3" t="str">
-        <v>5-7 Jahre</v>
-      </c>
-      <c r="I3" t="str">
-        <v>Schweiz</v>
-      </c>
       <c r="J3" t="str">
+        <v>Bachelor</v>
+      </c>
+      <c r="K3" t="str">
+        <v>Schweiz</v>
+      </c>
+      <c r="L3" t="str">
         <v>9000</v>
       </c>
     </row>
@@ -512,30 +532,36 @@
         <v>3</v>
       </c>
       <c r="B4" t="str">
-        <v>CEM (Customer Experience Manager)</v>
+        <v>Customer Experience Manager</v>
       </c>
       <c r="C4" t="str">
+        <v>Verantwortet die End-to-End-Customer-Journey und sorgt für konsistente, positive Kundenerlebnisse über alle Touchpoints. Analysiert Feedback, NPS und Verhaltensdaten, um Reibungspunkte zu reduzieren und Kundenbindung zu stärken. Arbeitet eng mit Marketing, Vertrieb und Service zusammen, um Prozesse kundenzentriert zu gestalten.</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Empathisch, datenaffin, prozessorientiert, kommunikativ, lösungsorientiert.</v>
+      </c>
+      <c r="E4" t="str">
+        <v>CRM-Tools (Salesforce, HubSpot), Customer-Journey-Mapping, NPS- und VoC-Programme, Cross-Functional Workshops.</v>
+      </c>
+      <c r="F4" t="str">
         <v>Weiblich</v>
       </c>
-      <c r="D4" t="str">
-        <v>20-29 Jahre</v>
-      </c>
-      <c r="E4" t="str">
-        <v>Schweiz</v>
-      </c>
-      <c r="F4" t="str">
+      <c r="G4" t="str">
+        <v>20-29 Jahre</v>
+      </c>
+      <c r="H4" t="str">
+        <v>Schweiz</v>
+      </c>
+      <c r="I4" t="str">
         <v>1 Person kein Kind</v>
       </c>
-      <c r="G4" t="str">
-        <v>Bachelor</v>
-      </c>
-      <c r="H4" t="str">
-        <v>5-7 Jahre</v>
-      </c>
-      <c r="I4" t="str">
-        <v>Schweiz</v>
-      </c>
       <c r="J4" t="str">
+        <v>Bachelor</v>
+      </c>
+      <c r="K4" t="str">
+        <v>Schweiz</v>
+      </c>
+      <c r="L4" t="str">
         <v>9000</v>
       </c>
     </row>
@@ -544,30 +570,36 @@
         <v>4</v>
       </c>
       <c r="B5" t="str">
-        <v>CEM (Customer Experience Manager)</v>
+        <v>Customer Experience Manager</v>
       </c>
       <c r="C5" t="str">
+        <v>Verantwortet die End-to-End-Customer-Journey und sorgt für konsistente, positive Kundenerlebnisse über alle Touchpoints. Analysiert Feedback, NPS und Verhaltensdaten, um Reibungspunkte zu reduzieren und Kundenbindung zu stärken. Arbeitet eng mit Marketing, Vertrieb und Service zusammen, um Prozesse kundenzentriert zu gestalten.</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Empathisch, datenaffin, prozessorientiert, kommunikativ, lösungsorientiert.</v>
+      </c>
+      <c r="E5" t="str">
+        <v>CRM-Tools (Salesforce, HubSpot), Customer-Journey-Mapping, NPS- und VoC-Programme, Cross-Functional Workshops.</v>
+      </c>
+      <c r="F5" t="str">
         <v>Weiblich</v>
       </c>
-      <c r="D5" t="str">
-        <v>20-29 Jahre</v>
-      </c>
-      <c r="E5" t="str">
-        <v>Schweiz</v>
-      </c>
-      <c r="F5" t="str">
+      <c r="G5" t="str">
+        <v>20-29 Jahre</v>
+      </c>
+      <c r="H5" t="str">
+        <v>Schweiz</v>
+      </c>
+      <c r="I5" t="str">
         <v>2 Personen 1 Kind</v>
       </c>
-      <c r="G5" t="str">
-        <v>Bachelor</v>
-      </c>
-      <c r="H5" t="str">
-        <v>5-7 Jahre</v>
-      </c>
-      <c r="I5" t="str">
-        <v>Schweiz</v>
-      </c>
       <c r="J5" t="str">
+        <v>Bachelor</v>
+      </c>
+      <c r="K5" t="str">
+        <v>Schweiz</v>
+      </c>
+      <c r="L5" t="str">
         <v>9000</v>
       </c>
     </row>
@@ -576,30 +608,36 @@
         <v>5</v>
       </c>
       <c r="B6" t="str">
-        <v>SMM (Social Media Manager)</v>
+        <v>Social Media Manager</v>
       </c>
       <c r="C6" t="str">
+        <v>Plant, erstellt und veröffentlicht Inhalte auf Social-Media-Kanälen und steuert das Community-Management. Beobachtet Trends, KPIs und Reichweiten, um Content-Strategien laufend zu optimieren. Setzt Paid- und Organic-Kampagnen zur Markenstärkung und Lead-Generierung um.</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Kreativ, trendbewusst, kommunikativ, schnell reagierend, analytisch.</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Instagram, TikTok, LinkedIn, Canva, Meta Business Suite, Hootsuite, Storytelling-Formate.</v>
+      </c>
+      <c r="F6" t="str">
         <v>Männlich</v>
       </c>
-      <c r="D6" t="str">
-        <v>20-29 Jahre</v>
-      </c>
-      <c r="E6" t="str">
-        <v>Schweiz</v>
-      </c>
-      <c r="F6" t="str">
+      <c r="G6" t="str">
+        <v>20-29 Jahre</v>
+      </c>
+      <c r="H6" t="str">
+        <v>Schweiz</v>
+      </c>
+      <c r="I6" t="str">
         <v>1 Person kein Kind</v>
       </c>
-      <c r="G6" t="str">
-        <v>Bachelor</v>
-      </c>
-      <c r="H6" t="str">
-        <v>2-5 Jahre</v>
-      </c>
-      <c r="I6" t="str">
-        <v>Schweiz</v>
-      </c>
       <c r="J6" t="str">
+        <v>Bachelor</v>
+      </c>
+      <c r="K6" t="str">
+        <v>Schweiz</v>
+      </c>
+      <c r="L6" t="str">
         <v>9000</v>
       </c>
     </row>
@@ -608,30 +646,36 @@
         <v>6</v>
       </c>
       <c r="B7" t="str">
-        <v>SMM (Social Media Manager)</v>
+        <v>Social Media Manager</v>
       </c>
       <c r="C7" t="str">
+        <v>Plant, erstellt und veröffentlicht Inhalte auf Social-Media-Kanälen und steuert das Community-Management. Beobachtet Trends, KPIs und Reichweiten, um Content-Strategien laufend zu optimieren. Setzt Paid- und Organic-Kampagnen zur Markenstärkung und Lead-Generierung um.</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Kreativ, trendbewusst, kommunikativ, schnell reagierend, analytisch.</v>
+      </c>
+      <c r="E7" t="str">
+        <v>Instagram, TikTok, LinkedIn, Canva, Meta Business Suite, Hootsuite, Storytelling-Formate.</v>
+      </c>
+      <c r="F7" t="str">
         <v>Männlich</v>
       </c>
-      <c r="D7" t="str">
-        <v>20-29 Jahre</v>
-      </c>
-      <c r="E7" t="str">
-        <v>Schweiz</v>
-      </c>
-      <c r="F7" t="str">
+      <c r="G7" t="str">
+        <v>20-29 Jahre</v>
+      </c>
+      <c r="H7" t="str">
+        <v>Schweiz</v>
+      </c>
+      <c r="I7" t="str">
         <v>2 Personen 1 Kind</v>
       </c>
-      <c r="G7" t="str">
-        <v>Bachelor</v>
-      </c>
-      <c r="H7" t="str">
-        <v>2-5 Jahre</v>
-      </c>
-      <c r="I7" t="str">
-        <v>Schweiz</v>
-      </c>
       <c r="J7" t="str">
+        <v>Bachelor</v>
+      </c>
+      <c r="K7" t="str">
+        <v>Schweiz</v>
+      </c>
+      <c r="L7" t="str">
         <v>9000</v>
       </c>
     </row>
@@ -640,30 +684,36 @@
         <v>7</v>
       </c>
       <c r="B8" t="str">
-        <v>SMM (Social Media Manager)</v>
+        <v>Social Media Manager</v>
       </c>
       <c r="C8" t="str">
+        <v>Plant, erstellt und veröffentlicht Inhalte auf Social-Media-Kanälen und steuert das Community-Management. Beobachtet Trends, KPIs und Reichweiten, um Content-Strategien laufend zu optimieren. Setzt Paid- und Organic-Kampagnen zur Markenstärkung und Lead-Generierung um.</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Kreativ, trendbewusst, kommunikativ, schnell reagierend, analytisch.</v>
+      </c>
+      <c r="E8" t="str">
+        <v>Instagram, TikTok, LinkedIn, Canva, Meta Business Suite, Hootsuite, Storytelling-Formate.</v>
+      </c>
+      <c r="F8" t="str">
         <v>Weiblich</v>
       </c>
-      <c r="D8" t="str">
-        <v>20-29 Jahre</v>
-      </c>
-      <c r="E8" t="str">
-        <v>Schweiz</v>
-      </c>
-      <c r="F8" t="str">
+      <c r="G8" t="str">
+        <v>20-29 Jahre</v>
+      </c>
+      <c r="H8" t="str">
+        <v>Schweiz</v>
+      </c>
+      <c r="I8" t="str">
         <v>1 Person kein Kind</v>
       </c>
-      <c r="G8" t="str">
-        <v>Bachelor</v>
-      </c>
-      <c r="H8" t="str">
-        <v>2-5 Jahre</v>
-      </c>
-      <c r="I8" t="str">
-        <v>Schweiz</v>
-      </c>
       <c r="J8" t="str">
+        <v>Bachelor</v>
+      </c>
+      <c r="K8" t="str">
+        <v>Schweiz</v>
+      </c>
+      <c r="L8" t="str">
         <v>9000</v>
       </c>
     </row>
@@ -672,30 +722,36 @@
         <v>8</v>
       </c>
       <c r="B9" t="str">
-        <v>SMM (Social Media Manager)</v>
+        <v>Social Media Manager</v>
       </c>
       <c r="C9" t="str">
+        <v>Plant, erstellt und veröffentlicht Inhalte auf Social-Media-Kanälen und steuert das Community-Management. Beobachtet Trends, KPIs und Reichweiten, um Content-Strategien laufend zu optimieren. Setzt Paid- und Organic-Kampagnen zur Markenstärkung und Lead-Generierung um.</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Kreativ, trendbewusst, kommunikativ, schnell reagierend, analytisch.</v>
+      </c>
+      <c r="E9" t="str">
+        <v>Instagram, TikTok, LinkedIn, Canva, Meta Business Suite, Hootsuite, Storytelling-Formate.</v>
+      </c>
+      <c r="F9" t="str">
         <v>Weiblich</v>
       </c>
-      <c r="D9" t="str">
-        <v>20-29 Jahre</v>
-      </c>
-      <c r="E9" t="str">
-        <v>Schweiz</v>
-      </c>
-      <c r="F9" t="str">
+      <c r="G9" t="str">
+        <v>20-29 Jahre</v>
+      </c>
+      <c r="H9" t="str">
+        <v>Schweiz</v>
+      </c>
+      <c r="I9" t="str">
         <v>2 Personen 1 Kind</v>
       </c>
-      <c r="G9" t="str">
-        <v>Bachelor</v>
-      </c>
-      <c r="H9" t="str">
-        <v>2-5 Jahre</v>
-      </c>
-      <c r="I9" t="str">
-        <v>Schweiz</v>
-      </c>
       <c r="J9" t="str">
+        <v>Bachelor</v>
+      </c>
+      <c r="K9" t="str">
+        <v>Schweiz</v>
+      </c>
+      <c r="L9" t="str">
         <v>9000</v>
       </c>
     </row>
@@ -704,30 +760,36 @@
         <v>9</v>
       </c>
       <c r="B10" t="str">
-        <v>DMM (Digital Manager)</v>
+        <v>Digital Manager</v>
       </c>
       <c r="C10" t="str">
+        <v>Steuert digitale Kanäle und Massnahmen, um Marken sichtbar zu machen und die Online-Performance zu steigern. Verantwortet Strategie und Umsetzung von SEO, SEA, E-Mail, Display und Social Ads. Analysiert Performance-Daten und optimiert Budgets entlang des Funnels.</v>
+      </c>
+      <c r="D10" t="str">
+        <v>Strategisch, datengetrieben, neugierig, kanalübergreifend denkend, ergebnisorientiert.</v>
+      </c>
+      <c r="E10" t="str">
+        <v>Google Ads, GA4, Meta Ads, Marketing-Automation, A/B-Testing, KPI-Dashboards.</v>
+      </c>
+      <c r="F10" t="str">
         <v>Männlich</v>
       </c>
-      <c r="D10" t="str">
-        <v>20-29 Jahre</v>
-      </c>
-      <c r="E10" t="str">
-        <v>Schweiz</v>
-      </c>
-      <c r="F10" t="str">
+      <c r="G10" t="str">
+        <v>20-29 Jahre</v>
+      </c>
+      <c r="H10" t="str">
+        <v>Schweiz</v>
+      </c>
+      <c r="I10" t="str">
         <v>1 Person kein Kind</v>
       </c>
-      <c r="G10" t="str">
-        <v>Bachelor</v>
-      </c>
-      <c r="H10" t="str">
-        <v>2-4 Jahre</v>
-      </c>
-      <c r="I10" t="str">
-        <v>Schweiz</v>
-      </c>
       <c r="J10" t="str">
+        <v>Bachelor</v>
+      </c>
+      <c r="K10" t="str">
+        <v>Schweiz</v>
+      </c>
+      <c r="L10" t="str">
         <v>9000</v>
       </c>
     </row>
@@ -736,30 +798,36 @@
         <v>10</v>
       </c>
       <c r="B11" t="str">
-        <v>DMM (Digital Manager)</v>
+        <v>Digital Manager</v>
       </c>
       <c r="C11" t="str">
+        <v>Steuert digitale Kanäle und Massnahmen, um Marken sichtbar zu machen und die Online-Performance zu steigern. Verantwortet Strategie und Umsetzung von SEO, SEA, E-Mail, Display und Social Ads. Analysiert Performance-Daten und optimiert Budgets entlang des Funnels.</v>
+      </c>
+      <c r="D11" t="str">
+        <v>Strategisch, datengetrieben, neugierig, kanalübergreifend denkend, ergebnisorientiert.</v>
+      </c>
+      <c r="E11" t="str">
+        <v>Google Ads, GA4, Meta Ads, Marketing-Automation, A/B-Testing, KPI-Dashboards.</v>
+      </c>
+      <c r="F11" t="str">
         <v>Männlich</v>
       </c>
-      <c r="D11" t="str">
-        <v>20-29 Jahre</v>
-      </c>
-      <c r="E11" t="str">
-        <v>Schweiz</v>
-      </c>
-      <c r="F11" t="str">
+      <c r="G11" t="str">
+        <v>20-29 Jahre</v>
+      </c>
+      <c r="H11" t="str">
+        <v>Schweiz</v>
+      </c>
+      <c r="I11" t="str">
         <v>2 Personen 1 Kind</v>
       </c>
-      <c r="G11" t="str">
-        <v>Bachelor</v>
-      </c>
-      <c r="H11" t="str">
-        <v>2-4 Jahre</v>
-      </c>
-      <c r="I11" t="str">
-        <v>Schweiz</v>
-      </c>
       <c r="J11" t="str">
+        <v>Bachelor</v>
+      </c>
+      <c r="K11" t="str">
+        <v>Schweiz</v>
+      </c>
+      <c r="L11" t="str">
         <v>9000</v>
       </c>
     </row>
@@ -768,30 +836,36 @@
         <v>11</v>
       </c>
       <c r="B12" t="str">
-        <v>DMM (Digital Manager)</v>
+        <v>Digital Manager</v>
       </c>
       <c r="C12" t="str">
+        <v>Steuert digitale Kanäle und Massnahmen, um Marken sichtbar zu machen und die Online-Performance zu steigern. Verantwortet Strategie und Umsetzung von SEO, SEA, E-Mail, Display und Social Ads. Analysiert Performance-Daten und optimiert Budgets entlang des Funnels.</v>
+      </c>
+      <c r="D12" t="str">
+        <v>Strategisch, datengetrieben, neugierig, kanalübergreifend denkend, ergebnisorientiert.</v>
+      </c>
+      <c r="E12" t="str">
+        <v>Google Ads, GA4, Meta Ads, Marketing-Automation, A/B-Testing, KPI-Dashboards.</v>
+      </c>
+      <c r="F12" t="str">
         <v>Weiblich</v>
       </c>
-      <c r="D12" t="str">
-        <v>20-29 Jahre</v>
-      </c>
-      <c r="E12" t="str">
-        <v>Schweiz</v>
-      </c>
-      <c r="F12" t="str">
+      <c r="G12" t="str">
+        <v>20-29 Jahre</v>
+      </c>
+      <c r="H12" t="str">
+        <v>Schweiz</v>
+      </c>
+      <c r="I12" t="str">
         <v>1 Person kein Kind</v>
       </c>
-      <c r="G12" t="str">
-        <v>Bachelor</v>
-      </c>
-      <c r="H12" t="str">
-        <v>2-4 Jahre</v>
-      </c>
-      <c r="I12" t="str">
-        <v>Schweiz</v>
-      </c>
       <c r="J12" t="str">
+        <v>Bachelor</v>
+      </c>
+      <c r="K12" t="str">
+        <v>Schweiz</v>
+      </c>
+      <c r="L12" t="str">
         <v>9000</v>
       </c>
     </row>
@@ -800,30 +874,36 @@
         <v>12</v>
       </c>
       <c r="B13" t="str">
-        <v>DMM (Digital Manager)</v>
+        <v>Digital Manager</v>
       </c>
       <c r="C13" t="str">
+        <v>Steuert digitale Kanäle und Massnahmen, um Marken sichtbar zu machen und die Online-Performance zu steigern. Verantwortet Strategie und Umsetzung von SEO, SEA, E-Mail, Display und Social Ads. Analysiert Performance-Daten und optimiert Budgets entlang des Funnels.</v>
+      </c>
+      <c r="D13" t="str">
+        <v>Strategisch, datengetrieben, neugierig, kanalübergreifend denkend, ergebnisorientiert.</v>
+      </c>
+      <c r="E13" t="str">
+        <v>Google Ads, GA4, Meta Ads, Marketing-Automation, A/B-Testing, KPI-Dashboards.</v>
+      </c>
+      <c r="F13" t="str">
         <v>Weiblich</v>
       </c>
-      <c r="D13" t="str">
-        <v>20-29 Jahre</v>
-      </c>
-      <c r="E13" t="str">
-        <v>Schweiz</v>
-      </c>
-      <c r="F13" t="str">
+      <c r="G13" t="str">
+        <v>20-29 Jahre</v>
+      </c>
+      <c r="H13" t="str">
+        <v>Schweiz</v>
+      </c>
+      <c r="I13" t="str">
         <v>2 Personen 1 Kind</v>
       </c>
-      <c r="G13" t="str">
-        <v>Bachelor</v>
-      </c>
-      <c r="H13" t="str">
-        <v>2-4 Jahre</v>
-      </c>
-      <c r="I13" t="str">
-        <v>Schweiz</v>
-      </c>
       <c r="J13" t="str">
+        <v>Bachelor</v>
+      </c>
+      <c r="K13" t="str">
+        <v>Schweiz</v>
+      </c>
+      <c r="L13" t="str">
         <v>9000</v>
       </c>
     </row>
@@ -835,27 +915,33 @@
         <v>Growth Manager</v>
       </c>
       <c r="C14" t="str">
+        <v>Treibt skalierbares Nutzer- und Umsatzwachstum durch experimentelle Massnahmen entlang des gesamten Funnels. Nutzt Daten, Hypothesen und schnelle Tests, um Akquise, Aktivierung und Retention zu verbessern. Arbeitet eng mit Produkt, Marketing und Engineering zusammen.</v>
+      </c>
+      <c r="D14" t="str">
+        <v>Hypothesengetrieben, experimentierfreudig, analytisch, technisch versiert, ergebnisfokussiert.</v>
+      </c>
+      <c r="E14" t="str">
+        <v>Mixpanel, Amplitude, GrowthBook, A/B-Testing, SQL, North-Star-Metriken, Lean-Experimente.</v>
+      </c>
+      <c r="F14" t="str">
         <v>Männlich</v>
       </c>
-      <c r="D14" t="str">
-        <v>20-29 Jahre</v>
-      </c>
-      <c r="E14" t="str">
-        <v>Schweiz</v>
-      </c>
-      <c r="F14" t="str">
+      <c r="G14" t="str">
+        <v>20-29 Jahre</v>
+      </c>
+      <c r="H14" t="str">
+        <v>Schweiz</v>
+      </c>
+      <c r="I14" t="str">
         <v>1 Person kein Kind</v>
       </c>
-      <c r="G14" t="str">
-        <v>Bachelor</v>
-      </c>
-      <c r="H14" t="str">
-        <v>2-4 Jahre</v>
-      </c>
-      <c r="I14" t="str">
-        <v>Schweiz</v>
-      </c>
       <c r="J14" t="str">
+        <v>Bachelor</v>
+      </c>
+      <c r="K14" t="str">
+        <v>Schweiz</v>
+      </c>
+      <c r="L14" t="str">
         <v>9000</v>
       </c>
     </row>
@@ -867,27 +953,33 @@
         <v>Growth Manager</v>
       </c>
       <c r="C15" t="str">
+        <v>Treibt skalierbares Nutzer- und Umsatzwachstum durch experimentelle Massnahmen entlang des gesamten Funnels. Nutzt Daten, Hypothesen und schnelle Tests, um Akquise, Aktivierung und Retention zu verbessern. Arbeitet eng mit Produkt, Marketing und Engineering zusammen.</v>
+      </c>
+      <c r="D15" t="str">
+        <v>Hypothesengetrieben, experimentierfreudig, analytisch, technisch versiert, ergebnisfokussiert.</v>
+      </c>
+      <c r="E15" t="str">
+        <v>Mixpanel, Amplitude, GrowthBook, A/B-Testing, SQL, North-Star-Metriken, Lean-Experimente.</v>
+      </c>
+      <c r="F15" t="str">
         <v>Männlich</v>
       </c>
-      <c r="D15" t="str">
-        <v>20-29 Jahre</v>
-      </c>
-      <c r="E15" t="str">
-        <v>Schweiz</v>
-      </c>
-      <c r="F15" t="str">
+      <c r="G15" t="str">
+        <v>20-29 Jahre</v>
+      </c>
+      <c r="H15" t="str">
+        <v>Schweiz</v>
+      </c>
+      <c r="I15" t="str">
         <v>2 Personen 1 Kind</v>
       </c>
-      <c r="G15" t="str">
-        <v>Bachelor</v>
-      </c>
-      <c r="H15" t="str">
-        <v>2-4 Jahre</v>
-      </c>
-      <c r="I15" t="str">
-        <v>Schweiz</v>
-      </c>
       <c r="J15" t="str">
+        <v>Bachelor</v>
+      </c>
+      <c r="K15" t="str">
+        <v>Schweiz</v>
+      </c>
+      <c r="L15" t="str">
         <v>9000</v>
       </c>
     </row>
@@ -899,27 +991,33 @@
         <v>Growth Manager</v>
       </c>
       <c r="C16" t="str">
+        <v>Treibt skalierbares Nutzer- und Umsatzwachstum durch experimentelle Massnahmen entlang des gesamten Funnels. Nutzt Daten, Hypothesen und schnelle Tests, um Akquise, Aktivierung und Retention zu verbessern. Arbeitet eng mit Produkt, Marketing und Engineering zusammen.</v>
+      </c>
+      <c r="D16" t="str">
+        <v>Hypothesengetrieben, experimentierfreudig, analytisch, technisch versiert, ergebnisfokussiert.</v>
+      </c>
+      <c r="E16" t="str">
+        <v>Mixpanel, Amplitude, GrowthBook, A/B-Testing, SQL, North-Star-Metriken, Lean-Experimente.</v>
+      </c>
+      <c r="F16" t="str">
         <v>Weiblich</v>
       </c>
-      <c r="D16" t="str">
-        <v>20-29 Jahre</v>
-      </c>
-      <c r="E16" t="str">
-        <v>Schweiz</v>
-      </c>
-      <c r="F16" t="str">
+      <c r="G16" t="str">
+        <v>20-29 Jahre</v>
+      </c>
+      <c r="H16" t="str">
+        <v>Schweiz</v>
+      </c>
+      <c r="I16" t="str">
         <v>1 Person kein Kind</v>
       </c>
-      <c r="G16" t="str">
-        <v>Bachelor</v>
-      </c>
-      <c r="H16" t="str">
-        <v>2-4 Jahre</v>
-      </c>
-      <c r="I16" t="str">
-        <v>Schweiz</v>
-      </c>
       <c r="J16" t="str">
+        <v>Bachelor</v>
+      </c>
+      <c r="K16" t="str">
+        <v>Schweiz</v>
+      </c>
+      <c r="L16" t="str">
         <v>9000</v>
       </c>
     </row>
@@ -931,27 +1029,33 @@
         <v>Growth Manager</v>
       </c>
       <c r="C17" t="str">
+        <v>Treibt skalierbares Nutzer- und Umsatzwachstum durch experimentelle Massnahmen entlang des gesamten Funnels. Nutzt Daten, Hypothesen und schnelle Tests, um Akquise, Aktivierung und Retention zu verbessern. Arbeitet eng mit Produkt, Marketing und Engineering zusammen.</v>
+      </c>
+      <c r="D17" t="str">
+        <v>Hypothesengetrieben, experimentierfreudig, analytisch, technisch versiert, ergebnisfokussiert.</v>
+      </c>
+      <c r="E17" t="str">
+        <v>Mixpanel, Amplitude, GrowthBook, A/B-Testing, SQL, North-Star-Metriken, Lean-Experimente.</v>
+      </c>
+      <c r="F17" t="str">
         <v>Weiblich</v>
       </c>
-      <c r="D17" t="str">
-        <v>20-29 Jahre</v>
-      </c>
-      <c r="E17" t="str">
-        <v>Schweiz</v>
-      </c>
-      <c r="F17" t="str">
+      <c r="G17" t="str">
+        <v>20-29 Jahre</v>
+      </c>
+      <c r="H17" t="str">
+        <v>Schweiz</v>
+      </c>
+      <c r="I17" t="str">
         <v>2 Personen 1 Kind</v>
       </c>
-      <c r="G17" t="str">
-        <v>Bachelor</v>
-      </c>
-      <c r="H17" t="str">
-        <v>2-4 Jahre</v>
-      </c>
-      <c r="I17" t="str">
-        <v>Schweiz</v>
-      </c>
       <c r="J17" t="str">
+        <v>Bachelor</v>
+      </c>
+      <c r="K17" t="str">
+        <v>Schweiz</v>
+      </c>
+      <c r="L17" t="str">
         <v>9000</v>
       </c>
     </row>
@@ -960,30 +1064,36 @@
         <v>17</v>
       </c>
       <c r="B18" t="str">
-        <v>Kommunikation Manager</v>
+        <v>Kommunikationsmanager</v>
       </c>
       <c r="C18" t="str">
+        <v>Verantwortet die interne und externe Kommunikation und sichert eine konsistente Markenstimme. Plant Pressemitteilungen, Statements, Krisenkommunikation und Stakeholder-Dialoge. Schreibt Inhalte, briefed Agenturen und steuert den Content-Kalender.</v>
+      </c>
+      <c r="D18" t="str">
+        <v>Sprachgewandt, strategisch, vertrauenswürdig, gut vernetzt, krisensicher.</v>
+      </c>
+      <c r="E18" t="str">
+        <v>PR-Tools, Newsroom-Plattformen, LinkedIn, klassische Medien, redaktionelle Workflows, Storytelling.</v>
+      </c>
+      <c r="F18" t="str">
         <v>Männlich</v>
       </c>
-      <c r="D18" t="str">
-        <v>20-29 Jahre</v>
-      </c>
-      <c r="E18" t="str">
-        <v>Schweiz</v>
-      </c>
-      <c r="F18" t="str">
+      <c r="G18" t="str">
+        <v>20-29 Jahre</v>
+      </c>
+      <c r="H18" t="str">
+        <v>Schweiz</v>
+      </c>
+      <c r="I18" t="str">
         <v>1 Person kein Kind</v>
       </c>
-      <c r="G18" t="str">
-        <v>Bachelor</v>
-      </c>
-      <c r="H18" t="str">
-        <v>4-6 Jahre</v>
-      </c>
-      <c r="I18" t="str">
-        <v>Schweiz</v>
-      </c>
       <c r="J18" t="str">
+        <v>Bachelor</v>
+      </c>
+      <c r="K18" t="str">
+        <v>Schweiz</v>
+      </c>
+      <c r="L18" t="str">
         <v>9000</v>
       </c>
     </row>
@@ -992,30 +1102,36 @@
         <v>18</v>
       </c>
       <c r="B19" t="str">
-        <v>Kommunikation Manager</v>
+        <v>Kommunikationsmanager</v>
       </c>
       <c r="C19" t="str">
+        <v>Verantwortet die interne und externe Kommunikation und sichert eine konsistente Markenstimme. Plant Pressemitteilungen, Statements, Krisenkommunikation und Stakeholder-Dialoge. Schreibt Inhalte, briefed Agenturen und steuert den Content-Kalender.</v>
+      </c>
+      <c r="D19" t="str">
+        <v>Sprachgewandt, strategisch, vertrauenswürdig, gut vernetzt, krisensicher.</v>
+      </c>
+      <c r="E19" t="str">
+        <v>PR-Tools, Newsroom-Plattformen, LinkedIn, klassische Medien, redaktionelle Workflows, Storytelling.</v>
+      </c>
+      <c r="F19" t="str">
         <v>Männlich</v>
       </c>
-      <c r="D19" t="str">
-        <v>20-29 Jahre</v>
-      </c>
-      <c r="E19" t="str">
-        <v>Schweiz</v>
-      </c>
-      <c r="F19" t="str">
+      <c r="G19" t="str">
+        <v>20-29 Jahre</v>
+      </c>
+      <c r="H19" t="str">
+        <v>Schweiz</v>
+      </c>
+      <c r="I19" t="str">
         <v>2 Personen 1 Kind</v>
       </c>
-      <c r="G19" t="str">
-        <v>Bachelor</v>
-      </c>
-      <c r="H19" t="str">
-        <v>4-6 Jahre</v>
-      </c>
-      <c r="I19" t="str">
-        <v>Schweiz</v>
-      </c>
       <c r="J19" t="str">
+        <v>Bachelor</v>
+      </c>
+      <c r="K19" t="str">
+        <v>Schweiz</v>
+      </c>
+      <c r="L19" t="str">
         <v>9000</v>
       </c>
     </row>
@@ -1024,30 +1140,36 @@
         <v>19</v>
       </c>
       <c r="B20" t="str">
-        <v>Kommunikation Manager</v>
+        <v>Kommunikationsmanager</v>
       </c>
       <c r="C20" t="str">
+        <v>Verantwortet die interne und externe Kommunikation und sichert eine konsistente Markenstimme. Plant Pressemitteilungen, Statements, Krisenkommunikation und Stakeholder-Dialoge. Schreibt Inhalte, briefed Agenturen und steuert den Content-Kalender.</v>
+      </c>
+      <c r="D20" t="str">
+        <v>Sprachgewandt, strategisch, vertrauenswürdig, gut vernetzt, krisensicher.</v>
+      </c>
+      <c r="E20" t="str">
+        <v>PR-Tools, Newsroom-Plattformen, LinkedIn, klassische Medien, redaktionelle Workflows, Storytelling.</v>
+      </c>
+      <c r="F20" t="str">
         <v>Weiblich</v>
       </c>
-      <c r="D20" t="str">
-        <v>20-29 Jahre</v>
-      </c>
-      <c r="E20" t="str">
-        <v>Schweiz</v>
-      </c>
-      <c r="F20" t="str">
+      <c r="G20" t="str">
+        <v>20-29 Jahre</v>
+      </c>
+      <c r="H20" t="str">
+        <v>Schweiz</v>
+      </c>
+      <c r="I20" t="str">
         <v>1 Person kein Kind</v>
       </c>
-      <c r="G20" t="str">
-        <v>Bachelor</v>
-      </c>
-      <c r="H20" t="str">
-        <v>4-6 Jahre</v>
-      </c>
-      <c r="I20" t="str">
-        <v>Schweiz</v>
-      </c>
       <c r="J20" t="str">
+        <v>Bachelor</v>
+      </c>
+      <c r="K20" t="str">
+        <v>Schweiz</v>
+      </c>
+      <c r="L20" t="str">
         <v>9000</v>
       </c>
     </row>
@@ -1056,30 +1178,36 @@
         <v>20</v>
       </c>
       <c r="B21" t="str">
-        <v>Kommunikation Manager</v>
+        <v>Kommunikationsmanager</v>
       </c>
       <c r="C21" t="str">
+        <v>Verantwortet die interne und externe Kommunikation und sichert eine konsistente Markenstimme. Plant Pressemitteilungen, Statements, Krisenkommunikation und Stakeholder-Dialoge. Schreibt Inhalte, briefed Agenturen und steuert den Content-Kalender.</v>
+      </c>
+      <c r="D21" t="str">
+        <v>Sprachgewandt, strategisch, vertrauenswürdig, gut vernetzt, krisensicher.</v>
+      </c>
+      <c r="E21" t="str">
+        <v>PR-Tools, Newsroom-Plattformen, LinkedIn, klassische Medien, redaktionelle Workflows, Storytelling.</v>
+      </c>
+      <c r="F21" t="str">
         <v>Weiblich</v>
       </c>
-      <c r="D21" t="str">
-        <v>20-29 Jahre</v>
-      </c>
-      <c r="E21" t="str">
-        <v>Schweiz</v>
-      </c>
-      <c r="F21" t="str">
+      <c r="G21" t="str">
+        <v>20-29 Jahre</v>
+      </c>
+      <c r="H21" t="str">
+        <v>Schweiz</v>
+      </c>
+      <c r="I21" t="str">
         <v>2 Personen 1 Kind</v>
       </c>
-      <c r="G21" t="str">
-        <v>Bachelor</v>
-      </c>
-      <c r="H21" t="str">
-        <v>4-6 Jahre</v>
-      </c>
-      <c r="I21" t="str">
-        <v>Schweiz</v>
-      </c>
       <c r="J21" t="str">
+        <v>Bachelor</v>
+      </c>
+      <c r="K21" t="str">
+        <v>Schweiz</v>
+      </c>
+      <c r="L21" t="str">
         <v>9000</v>
       </c>
     </row>
@@ -1088,30 +1216,36 @@
         <v>21</v>
       </c>
       <c r="B22" t="str">
-        <v>Webseiten Manager</v>
+        <v>Website Manager</v>
       </c>
       <c r="C22" t="str">
+        <v>Verantwortet Konzeption, Pflege und Weiterentwicklung der Unternehmenswebsite. Überwacht Performance, SEO, UX und Conversion und steuert Anpassungen mit Entwicklung und Design. Sorgt für rechtssichere, barrierearme Inhalte und einen reibungslosen technischen Betrieb.</v>
+      </c>
+      <c r="D22" t="str">
+        <v>Detailgenau, technisch versiert, UX-affin, strukturiert, datengetrieben.</v>
+      </c>
+      <c r="E22" t="str">
+        <v>CMS (WordPress, Webflow, TYPO3), GA4, Search Console, Lighthouse, A/B-Testing, Figma.</v>
+      </c>
+      <c r="F22" t="str">
         <v>Männlich</v>
       </c>
-      <c r="D22" t="str">
-        <v>20-29 Jahre</v>
-      </c>
-      <c r="E22" t="str">
-        <v>Schweiz</v>
-      </c>
-      <c r="F22" t="str">
+      <c r="G22" t="str">
+        <v>20-29 Jahre</v>
+      </c>
+      <c r="H22" t="str">
+        <v>Schweiz</v>
+      </c>
+      <c r="I22" t="str">
         <v>1 Person kein Kind</v>
       </c>
-      <c r="G22" t="str">
-        <v>Bachelor</v>
-      </c>
-      <c r="H22" t="str">
-        <v>5-7 Jahre</v>
-      </c>
-      <c r="I22" t="str">
-        <v>Schweiz</v>
-      </c>
       <c r="J22" t="str">
+        <v>Bachelor</v>
+      </c>
+      <c r="K22" t="str">
+        <v>Schweiz</v>
+      </c>
+      <c r="L22" t="str">
         <v>9000</v>
       </c>
     </row>
@@ -1120,30 +1254,36 @@
         <v>22</v>
       </c>
       <c r="B23" t="str">
-        <v>Webseiten Manager</v>
+        <v>Website Manager</v>
       </c>
       <c r="C23" t="str">
+        <v>Verantwortet Konzeption, Pflege und Weiterentwicklung der Unternehmenswebsite. Überwacht Performance, SEO, UX und Conversion und steuert Anpassungen mit Entwicklung und Design. Sorgt für rechtssichere, barrierearme Inhalte und einen reibungslosen technischen Betrieb.</v>
+      </c>
+      <c r="D23" t="str">
+        <v>Detailgenau, technisch versiert, UX-affin, strukturiert, datengetrieben.</v>
+      </c>
+      <c r="E23" t="str">
+        <v>CMS (WordPress, Webflow, TYPO3), GA4, Search Console, Lighthouse, A/B-Testing, Figma.</v>
+      </c>
+      <c r="F23" t="str">
         <v>Männlich</v>
       </c>
-      <c r="D23" t="str">
-        <v>20-29 Jahre</v>
-      </c>
-      <c r="E23" t="str">
-        <v>Schweiz</v>
-      </c>
-      <c r="F23" t="str">
+      <c r="G23" t="str">
+        <v>20-29 Jahre</v>
+      </c>
+      <c r="H23" t="str">
+        <v>Schweiz</v>
+      </c>
+      <c r="I23" t="str">
         <v>2 Personen 1 Kind</v>
       </c>
-      <c r="G23" t="str">
-        <v>Bachelor</v>
-      </c>
-      <c r="H23" t="str">
-        <v>5-7 Jahre</v>
-      </c>
-      <c r="I23" t="str">
-        <v>Schweiz</v>
-      </c>
       <c r="J23" t="str">
+        <v>Bachelor</v>
+      </c>
+      <c r="K23" t="str">
+        <v>Schweiz</v>
+      </c>
+      <c r="L23" t="str">
         <v>9000</v>
       </c>
     </row>
@@ -1152,30 +1292,36 @@
         <v>23</v>
       </c>
       <c r="B24" t="str">
-        <v>Webseiten Manager</v>
+        <v>Website Manager</v>
       </c>
       <c r="C24" t="str">
+        <v>Verantwortet Konzeption, Pflege und Weiterentwicklung der Unternehmenswebsite. Überwacht Performance, SEO, UX und Conversion und steuert Anpassungen mit Entwicklung und Design. Sorgt für rechtssichere, barrierearme Inhalte und einen reibungslosen technischen Betrieb.</v>
+      </c>
+      <c r="D24" t="str">
+        <v>Detailgenau, technisch versiert, UX-affin, strukturiert, datengetrieben.</v>
+      </c>
+      <c r="E24" t="str">
+        <v>CMS (WordPress, Webflow, TYPO3), GA4, Search Console, Lighthouse, A/B-Testing, Figma.</v>
+      </c>
+      <c r="F24" t="str">
         <v>Weiblich</v>
       </c>
-      <c r="D24" t="str">
-        <v>20-29 Jahre</v>
-      </c>
-      <c r="E24" t="str">
-        <v>Schweiz</v>
-      </c>
-      <c r="F24" t="str">
+      <c r="G24" t="str">
+        <v>20-29 Jahre</v>
+      </c>
+      <c r="H24" t="str">
+        <v>Schweiz</v>
+      </c>
+      <c r="I24" t="str">
         <v>1 Person kein Kind</v>
       </c>
-      <c r="G24" t="str">
-        <v>Bachelor</v>
-      </c>
-      <c r="H24" t="str">
-        <v>5-7 Jahre</v>
-      </c>
-      <c r="I24" t="str">
-        <v>Schweiz</v>
-      </c>
       <c r="J24" t="str">
+        <v>Bachelor</v>
+      </c>
+      <c r="K24" t="str">
+        <v>Schweiz</v>
+      </c>
+      <c r="L24" t="str">
         <v>9000</v>
       </c>
     </row>
@@ -1184,36 +1330,42 @@
         <v>24</v>
       </c>
       <c r="B25" t="str">
-        <v>Webseiten Manager</v>
+        <v>Website Manager</v>
       </c>
       <c r="C25" t="str">
+        <v>Verantwortet Konzeption, Pflege und Weiterentwicklung der Unternehmenswebsite. Überwacht Performance, SEO, UX und Conversion und steuert Anpassungen mit Entwicklung und Design. Sorgt für rechtssichere, barrierearme Inhalte und einen reibungslosen technischen Betrieb.</v>
+      </c>
+      <c r="D25" t="str">
+        <v>Detailgenau, technisch versiert, UX-affin, strukturiert, datengetrieben.</v>
+      </c>
+      <c r="E25" t="str">
+        <v>CMS (WordPress, Webflow, TYPO3), GA4, Search Console, Lighthouse, A/B-Testing, Figma.</v>
+      </c>
+      <c r="F25" t="str">
         <v>Weiblich</v>
       </c>
-      <c r="D25" t="str">
-        <v>20-29 Jahre</v>
-      </c>
-      <c r="E25" t="str">
-        <v>Schweiz</v>
-      </c>
-      <c r="F25" t="str">
+      <c r="G25" t="str">
+        <v>20-29 Jahre</v>
+      </c>
+      <c r="H25" t="str">
+        <v>Schweiz</v>
+      </c>
+      <c r="I25" t="str">
         <v>2 Personen 1 Kind</v>
       </c>
-      <c r="G25" t="str">
-        <v>Bachelor</v>
-      </c>
-      <c r="H25" t="str">
-        <v>5-7 Jahre</v>
-      </c>
-      <c r="I25" t="str">
-        <v>Schweiz</v>
-      </c>
       <c r="J25" t="str">
+        <v>Bachelor</v>
+      </c>
+      <c r="K25" t="str">
+        <v>Schweiz</v>
+      </c>
+      <c r="L25" t="str">
         <v>9000</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J25"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L25"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Bundle role meta into single 'Avatar Eigenschaften und Praeferenzen' column
Restores the 24-row demografische Struktur und ersetzt die getrennte
Berufserfahrung-Spalte durch eine kombinierte Textspalte mit
Jobbezeichnung, Jobbeschreibung, Berufserfahrung und Avatar-Eigenschaften
(1:1 aus src/app/page.tsx).
</commit_message>
<xml_diff>
--- a/personas_24.xlsx
+++ b/personas_24.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Personas" sheetId="1" r:id="rId1"/>
+    <sheet name="Personas_24" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -397,115 +397,967 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:J25"/>
   <cols>
-    <col min="1" max="1" width="30.83203125" customWidth="1"/>
-    <col min="2" max="2" width="90.83203125" customWidth="1"/>
-    <col min="3" max="3" width="60.83203125" customWidth="1"/>
-    <col min="4" max="4" width="60.83203125" customWidth="1"/>
+    <col min="1" max="1" width="4.83203125" customWidth="1"/>
+    <col min="2" max="2" width="36.83203125" customWidth="1"/>
+    <col min="3" max="3" width="11.83203125" customWidth="1"/>
+    <col min="4" max="4" width="13.83203125" customWidth="1"/>
+    <col min="5" max="5" width="13.83203125" customWidth="1"/>
+    <col min="6" max="6" width="22.83203125" customWidth="1"/>
+    <col min="7" max="7" width="18.83203125" customWidth="1"/>
+    <col min="8" max="8" width="13.83203125" customWidth="1"/>
+    <col min="9" max="9" width="11.83203125" customWidth="1"/>
+    <col min="10" max="10" width="110.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Jobbezeichnung</v>
+        <v>ID</v>
       </c>
       <c r="B1" t="str">
-        <v>Jobbeschreibung</v>
+        <v>Rolle</v>
       </c>
       <c r="C1" t="str">
-        <v>Avatar Eigenschaften</v>
+        <v>Geschlecht</v>
       </c>
       <c r="D1" t="str">
-        <v>Präferenzen</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>Customer Experience Manager</v>
+        <v>Alter</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Nationalitaet</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Haushalt</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Ausbildung</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Wohnsitzland</v>
+      </c>
+      <c r="I1" t="str">
+        <v>Postleitzahl</v>
+      </c>
+      <c r="J1" t="str">
+        <v>Avatar Eigenschaften und Präferenzen</v>
+      </c>
+    </row>
+    <row r="2" xml:space="preserve">
+      <c r="A2">
+        <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v>Verantwortet die End-to-End-Customer-Journey und sorgt für konsistente, positive Kundenerlebnisse über alle Touchpoints. Analysiert Feedback, NPS und Verhaltensdaten, um Reibungspunkte zu reduzieren und Kundenbindung zu stärken. Arbeitet eng mit Marketing, Vertrieb und Service zusammen, um Prozesse kundenzentriert zu gestalten.</v>
+        <v>CEM (Customer Experience Manager)</v>
       </c>
       <c r="C2" t="str">
-        <v>Empathisch, datenaffin, prozessorientiert, kommunikativ, lösungsorientiert.</v>
+        <v>Männlich</v>
       </c>
       <c r="D2" t="str">
-        <v>CRM-Tools (Salesforce, HubSpot), Customer-Journey-Mapping, NPS- und VoC-Programme, Cross-Functional Workshops.</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>Social Media Manager</v>
+        <v>20-29 Jahre</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Schweiz</v>
+      </c>
+      <c r="F2" t="str">
+        <v>1 Person kein Kind</v>
+      </c>
+      <c r="G2" t="str">
+        <v>Bachelor</v>
+      </c>
+      <c r="H2" t="str">
+        <v>Schweiz</v>
+      </c>
+      <c r="I2" t="str">
+        <v>9000</v>
+      </c>
+      <c r="J2" t="str" xml:space="preserve">
+        <v xml:space="preserve">Jobbezeichnung: Customer Experience Manager
+Jobbeschreibung: Verantwortet die End-to-End-Customer-Journey und sorgt für konsistente, positive Kundenerlebnisse über alle Touchpoints. Analysiert Feedback, NPS und Verhaltensdaten, um Reibungspunkte zu reduzieren und Kundenbindung zu stärken. Arbeitet eng mit Marketing, Vertrieb und Service zusammen, um Prozesse kundenzentriert zu gestalten.
+Berufserfahrung: 5-7 Jahre
+Branchenwissen: Customer Experience, Customer Service, Marketing / Customer Relations
+Tools &amp; Technologien: Microsoft Office / Shopify, Microsoft PowerPoint / Marketing Automation (HubSpot/Klaviyo), Microsoft Excel / Google Ads / Google Marketing Suite
+Soziale Kompetenz: Teamwork / Structured working style, Leadership / Teamwork / Collaboration, Customer Service / Organizational skills
+Weitere Kenntnisse: Project Management / Customer Journey / UX, Event Management / Campaign Management, Analytical Skills / Präsentationsskills</v>
+      </c>
+    </row>
+    <row r="3" xml:space="preserve">
+      <c r="A3">
+        <v>2</v>
       </c>
       <c r="B3" t="str">
-        <v>Plant, erstellt und veröffentlicht Inhalte auf Social-Media-Kanälen und steuert das Community-Management. Beobachtet Trends, KPIs und Reichweiten, um Content-Strategien laufend zu optimieren. Setzt Paid- und Organic-Kampagnen zur Markenstärkung und Lead-Generierung um.</v>
+        <v>CEM (Customer Experience Manager)</v>
       </c>
       <c r="C3" t="str">
-        <v>Kreativ, trendbewusst, kommunikativ, schnell reagierend, analytisch.</v>
+        <v>Männlich</v>
       </c>
       <c r="D3" t="str">
-        <v>Instagram, TikTok, LinkedIn, Canva, Meta Business Suite, Hootsuite, Storytelling-Formate.</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>Digital Manager</v>
+        <v>20-29 Jahre</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Schweiz</v>
+      </c>
+      <c r="F3" t="str">
+        <v>2 Personen 1 Kind</v>
+      </c>
+      <c r="G3" t="str">
+        <v>Bachelor</v>
+      </c>
+      <c r="H3" t="str">
+        <v>Schweiz</v>
+      </c>
+      <c r="I3" t="str">
+        <v>9000</v>
+      </c>
+      <c r="J3" t="str" xml:space="preserve">
+        <v xml:space="preserve">Jobbezeichnung: Customer Experience Manager
+Jobbeschreibung: Verantwortet die End-to-End-Customer-Journey und sorgt für konsistente, positive Kundenerlebnisse über alle Touchpoints. Analysiert Feedback, NPS und Verhaltensdaten, um Reibungspunkte zu reduzieren und Kundenbindung zu stärken. Arbeitet eng mit Marketing, Vertrieb und Service zusammen, um Prozesse kundenzentriert zu gestalten.
+Berufserfahrung: 5-7 Jahre
+Branchenwissen: Customer Experience, Customer Service, Marketing / Customer Relations
+Tools &amp; Technologien: Microsoft Office / Shopify, Microsoft PowerPoint / Marketing Automation (HubSpot/Klaviyo), Microsoft Excel / Google Ads / Google Marketing Suite
+Soziale Kompetenz: Teamwork / Structured working style, Leadership / Teamwork / Collaboration, Customer Service / Organizational skills
+Weitere Kenntnisse: Project Management / Customer Journey / UX, Event Management / Campaign Management, Analytical Skills / Präsentationsskills</v>
+      </c>
+    </row>
+    <row r="4" xml:space="preserve">
+      <c r="A4">
+        <v>3</v>
       </c>
       <c r="B4" t="str">
-        <v>Steuert digitale Kanäle und Massnahmen, um Marken sichtbar zu machen und die Online-Performance zu steigern. Verantwortet Strategie und Umsetzung von SEO, SEA, E-Mail, Display und Social Ads. Analysiert Performance-Daten und optimiert Budgets entlang des Funnels.</v>
+        <v>CEM (Customer Experience Manager)</v>
       </c>
       <c r="C4" t="str">
-        <v>Strategisch, datengetrieben, neugierig, kanalübergreifend denkend, ergebnisorientiert.</v>
+        <v>Weiblich</v>
       </c>
       <c r="D4" t="str">
-        <v>Google Ads, GA4, Meta Ads, Marketing-Automation, A/B-Testing, KPI-Dashboards.</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
+        <v>20-29 Jahre</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Schweiz</v>
+      </c>
+      <c r="F4" t="str">
+        <v>1 Person kein Kind</v>
+      </c>
+      <c r="G4" t="str">
+        <v>Bachelor</v>
+      </c>
+      <c r="H4" t="str">
+        <v>Schweiz</v>
+      </c>
+      <c r="I4" t="str">
+        <v>9000</v>
+      </c>
+      <c r="J4" t="str" xml:space="preserve">
+        <v xml:space="preserve">Jobbezeichnung: Customer Experience Manager
+Jobbeschreibung: Verantwortet die End-to-End-Customer-Journey und sorgt für konsistente, positive Kundenerlebnisse über alle Touchpoints. Analysiert Feedback, NPS und Verhaltensdaten, um Reibungspunkte zu reduzieren und Kundenbindung zu stärken. Arbeitet eng mit Marketing, Vertrieb und Service zusammen, um Prozesse kundenzentriert zu gestalten.
+Berufserfahrung: 5-7 Jahre
+Branchenwissen: Customer Experience, Customer Service, Marketing / Customer Relations
+Tools &amp; Technologien: Microsoft Office / Shopify, Microsoft PowerPoint / Marketing Automation (HubSpot/Klaviyo), Microsoft Excel / Google Ads / Google Marketing Suite
+Soziale Kompetenz: Teamwork / Structured working style, Leadership / Teamwork / Collaboration, Customer Service / Organizational skills
+Weitere Kenntnisse: Project Management / Customer Journey / UX, Event Management / Campaign Management, Analytical Skills / Präsentationsskills</v>
+      </c>
+    </row>
+    <row r="5" xml:space="preserve">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="str">
+        <v>CEM (Customer Experience Manager)</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Weiblich</v>
+      </c>
+      <c r="D5" t="str">
+        <v>20-29 Jahre</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Schweiz</v>
+      </c>
+      <c r="F5" t="str">
+        <v>2 Personen 1 Kind</v>
+      </c>
+      <c r="G5" t="str">
+        <v>Bachelor</v>
+      </c>
+      <c r="H5" t="str">
+        <v>Schweiz</v>
+      </c>
+      <c r="I5" t="str">
+        <v>9000</v>
+      </c>
+      <c r="J5" t="str" xml:space="preserve">
+        <v xml:space="preserve">Jobbezeichnung: Customer Experience Manager
+Jobbeschreibung: Verantwortet die End-to-End-Customer-Journey und sorgt für konsistente, positive Kundenerlebnisse über alle Touchpoints. Analysiert Feedback, NPS und Verhaltensdaten, um Reibungspunkte zu reduzieren und Kundenbindung zu stärken. Arbeitet eng mit Marketing, Vertrieb und Service zusammen, um Prozesse kundenzentriert zu gestalten.
+Berufserfahrung: 5-7 Jahre
+Branchenwissen: Customer Experience, Customer Service, Marketing / Customer Relations
+Tools &amp; Technologien: Microsoft Office / Shopify, Microsoft PowerPoint / Marketing Automation (HubSpot/Klaviyo), Microsoft Excel / Google Ads / Google Marketing Suite
+Soziale Kompetenz: Teamwork / Structured working style, Leadership / Teamwork / Collaboration, Customer Service / Organizational skills
+Weitere Kenntnisse: Project Management / Customer Journey / UX, Event Management / Campaign Management, Analytical Skills / Präsentationsskills</v>
+      </c>
+    </row>
+    <row r="6" xml:space="preserve">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="str">
+        <v>SMM (Social Media Manager)</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Männlich</v>
+      </c>
+      <c r="D6" t="str">
+        <v>20-29 Jahre</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Schweiz</v>
+      </c>
+      <c r="F6" t="str">
+        <v>1 Person kein Kind</v>
+      </c>
+      <c r="G6" t="str">
+        <v>Bachelor</v>
+      </c>
+      <c r="H6" t="str">
+        <v>Schweiz</v>
+      </c>
+      <c r="I6" t="str">
+        <v>9000</v>
+      </c>
+      <c r="J6" t="str" xml:space="preserve">
+        <v xml:space="preserve">Jobbezeichnung: Social Media Manager
+Jobbeschreibung: Plant, erstellt und veröffentlicht Inhalte auf Social-Media-Kanälen und steuert das Community-Management. Beobachtet Trends, KPIs und Reichweiten, um Content-Strategien laufend zu optimieren. Setzt Paid- und Organic-Kampagnen zur Markenstärkung und Lead-Generierung um.
+Berufserfahrung: 2-5 Jahre
+Branchenwissen: Digital Marketing, Marketing, E-Commerce
+Tools &amp; Technologien: Microsoft Office / Analytics &amp; BI (Tableau/Looker/Power BI), Google Analytics / CMS (WordPress/Typo3/other), Microsoft Excel / Google Ads / Google Marketing Suite
+Soziale Kompetenz: Teamwork / Teamwork / Collaboration, Communication / Analytical thinking, Project Management / Proactive / autonomous working style
+Weitere Kenntnisse: Project Management / Campaign Management, Online Marketing / KPI / Analytics &amp; Reporting, Social Media / Performance Marketing</v>
+      </c>
+    </row>
+    <row r="7" xml:space="preserve">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" t="str">
+        <v>SMM (Social Media Manager)</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Männlich</v>
+      </c>
+      <c r="D7" t="str">
+        <v>20-29 Jahre</v>
+      </c>
+      <c r="E7" t="str">
+        <v>Schweiz</v>
+      </c>
+      <c r="F7" t="str">
+        <v>2 Personen 1 Kind</v>
+      </c>
+      <c r="G7" t="str">
+        <v>Bachelor</v>
+      </c>
+      <c r="H7" t="str">
+        <v>Schweiz</v>
+      </c>
+      <c r="I7" t="str">
+        <v>9000</v>
+      </c>
+      <c r="J7" t="str" xml:space="preserve">
+        <v xml:space="preserve">Jobbezeichnung: Social Media Manager
+Jobbeschreibung: Plant, erstellt und veröffentlicht Inhalte auf Social-Media-Kanälen und steuert das Community-Management. Beobachtet Trends, KPIs und Reichweiten, um Content-Strategien laufend zu optimieren. Setzt Paid- und Organic-Kampagnen zur Markenstärkung und Lead-Generierung um.
+Berufserfahrung: 2-5 Jahre
+Branchenwissen: Digital Marketing, Marketing, E-Commerce
+Tools &amp; Technologien: Microsoft Office / Analytics &amp; BI (Tableau/Looker/Power BI), Google Analytics / CMS (WordPress/Typo3/other), Microsoft Excel / Google Ads / Google Marketing Suite
+Soziale Kompetenz: Teamwork / Teamwork / Collaboration, Communication / Analytical thinking, Project Management / Proactive / autonomous working style
+Weitere Kenntnisse: Project Management / Campaign Management, Online Marketing / KPI / Analytics &amp; Reporting, Social Media / Performance Marketing</v>
+      </c>
+    </row>
+    <row r="8" xml:space="preserve">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" t="str">
+        <v>SMM (Social Media Manager)</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Weiblich</v>
+      </c>
+      <c r="D8" t="str">
+        <v>20-29 Jahre</v>
+      </c>
+      <c r="E8" t="str">
+        <v>Schweiz</v>
+      </c>
+      <c r="F8" t="str">
+        <v>1 Person kein Kind</v>
+      </c>
+      <c r="G8" t="str">
+        <v>Bachelor</v>
+      </c>
+      <c r="H8" t="str">
+        <v>Schweiz</v>
+      </c>
+      <c r="I8" t="str">
+        <v>9000</v>
+      </c>
+      <c r="J8" t="str" xml:space="preserve">
+        <v xml:space="preserve">Jobbezeichnung: Social Media Manager
+Jobbeschreibung: Plant, erstellt und veröffentlicht Inhalte auf Social-Media-Kanälen und steuert das Community-Management. Beobachtet Trends, KPIs und Reichweiten, um Content-Strategien laufend zu optimieren. Setzt Paid- und Organic-Kampagnen zur Markenstärkung und Lead-Generierung um.
+Berufserfahrung: 2-5 Jahre
+Branchenwissen: Digital Marketing, Marketing, E-Commerce
+Tools &amp; Technologien: Microsoft Office / Analytics &amp; BI (Tableau/Looker/Power BI), Google Analytics / CMS (WordPress/Typo3/other), Microsoft Excel / Google Ads / Google Marketing Suite
+Soziale Kompetenz: Teamwork / Teamwork / Collaboration, Communication / Analytical thinking, Project Management / Proactive / autonomous working style
+Weitere Kenntnisse: Project Management / Campaign Management, Online Marketing / KPI / Analytics &amp; Reporting, Social Media / Performance Marketing</v>
+      </c>
+    </row>
+    <row r="9" xml:space="preserve">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" t="str">
+        <v>SMM (Social Media Manager)</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Weiblich</v>
+      </c>
+      <c r="D9" t="str">
+        <v>20-29 Jahre</v>
+      </c>
+      <c r="E9" t="str">
+        <v>Schweiz</v>
+      </c>
+      <c r="F9" t="str">
+        <v>2 Personen 1 Kind</v>
+      </c>
+      <c r="G9" t="str">
+        <v>Bachelor</v>
+      </c>
+      <c r="H9" t="str">
+        <v>Schweiz</v>
+      </c>
+      <c r="I9" t="str">
+        <v>9000</v>
+      </c>
+      <c r="J9" t="str" xml:space="preserve">
+        <v xml:space="preserve">Jobbezeichnung: Social Media Manager
+Jobbeschreibung: Plant, erstellt und veröffentlicht Inhalte auf Social-Media-Kanälen und steuert das Community-Management. Beobachtet Trends, KPIs und Reichweiten, um Content-Strategien laufend zu optimieren. Setzt Paid- und Organic-Kampagnen zur Markenstärkung und Lead-Generierung um.
+Berufserfahrung: 2-5 Jahre
+Branchenwissen: Digital Marketing, Marketing, E-Commerce
+Tools &amp; Technologien: Microsoft Office / Analytics &amp; BI (Tableau/Looker/Power BI), Google Analytics / CMS (WordPress/Typo3/other), Microsoft Excel / Google Ads / Google Marketing Suite
+Soziale Kompetenz: Teamwork / Teamwork / Collaboration, Communication / Analytical thinking, Project Management / Proactive / autonomous working style
+Weitere Kenntnisse: Project Management / Campaign Management, Online Marketing / KPI / Analytics &amp; Reporting, Social Media / Performance Marketing</v>
+      </c>
+    </row>
+    <row r="10" xml:space="preserve">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" t="str">
+        <v>DMM (Digital Manager)</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Männlich</v>
+      </c>
+      <c r="D10" t="str">
+        <v>20-29 Jahre</v>
+      </c>
+      <c r="E10" t="str">
+        <v>Schweiz</v>
+      </c>
+      <c r="F10" t="str">
+        <v>1 Person kein Kind</v>
+      </c>
+      <c r="G10" t="str">
+        <v>Bachelor</v>
+      </c>
+      <c r="H10" t="str">
+        <v>Schweiz</v>
+      </c>
+      <c r="I10" t="str">
+        <v>9000</v>
+      </c>
+      <c r="J10" t="str" xml:space="preserve">
+        <v xml:space="preserve">Jobbezeichnung: Digital Manager
+Jobbeschreibung: Steuert digitale Kanäle und Massnahmen, um Marken sichtbar zu machen und die Online-Performance zu steigern. Verantwortet Strategie und Umsetzung von SEO, SEA, E-Mail, Display und Social Ads. Analysiert Performance-Daten und optimiert Budgets entlang des Funnels.
+Berufserfahrung: 2-4 Jahre
+Branchenwissen: Social Media Marketing / Content Creation, Digital Marketing / Kommunikation, Social Media / Partnerschaften
+Tools &amp; Technologien: Microsoft Office / Adobe Creative Suite, Microsoft PowerPoint / Social Media Platforms (FB/TikTok/IG), Microsoft Word / CMS / Typo3
+Soziale Kompetenz: Teamwork / Teamwork / Collaboration, Leadership / Structured working style, Communication / Proactive / autonomous
+Weitere Kenntnisse: Social Media / Social Media Strategy, Sales / Content Strategy &amp; Planning, Project Management / Video &amp; Photo Production</v>
+      </c>
+    </row>
+    <row r="11" xml:space="preserve">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" t="str">
+        <v>DMM (Digital Manager)</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Männlich</v>
+      </c>
+      <c r="D11" t="str">
+        <v>20-29 Jahre</v>
+      </c>
+      <c r="E11" t="str">
+        <v>Schweiz</v>
+      </c>
+      <c r="F11" t="str">
+        <v>2 Personen 1 Kind</v>
+      </c>
+      <c r="G11" t="str">
+        <v>Bachelor</v>
+      </c>
+      <c r="H11" t="str">
+        <v>Schweiz</v>
+      </c>
+      <c r="I11" t="str">
+        <v>9000</v>
+      </c>
+      <c r="J11" t="str" xml:space="preserve">
+        <v xml:space="preserve">Jobbezeichnung: Digital Manager
+Jobbeschreibung: Steuert digitale Kanäle und Massnahmen, um Marken sichtbar zu machen und die Online-Performance zu steigern. Verantwortet Strategie und Umsetzung von SEO, SEA, E-Mail, Display und Social Ads. Analysiert Performance-Daten und optimiert Budgets entlang des Funnels.
+Berufserfahrung: 2-4 Jahre
+Branchenwissen: Social Media Marketing / Content Creation, Digital Marketing / Kommunikation, Social Media / Partnerschaften
+Tools &amp; Technologien: Microsoft Office / Adobe Creative Suite, Microsoft PowerPoint / Social Media Platforms (FB/TikTok/IG), Microsoft Word / CMS / Typo3
+Soziale Kompetenz: Teamwork / Teamwork / Collaboration, Leadership / Structured working style, Communication / Proactive / autonomous
+Weitere Kenntnisse: Social Media / Social Media Strategy, Sales / Content Strategy &amp; Planning, Project Management / Video &amp; Photo Production</v>
+      </c>
+    </row>
+    <row r="12" xml:space="preserve">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" t="str">
+        <v>DMM (Digital Manager)</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Weiblich</v>
+      </c>
+      <c r="D12" t="str">
+        <v>20-29 Jahre</v>
+      </c>
+      <c r="E12" t="str">
+        <v>Schweiz</v>
+      </c>
+      <c r="F12" t="str">
+        <v>1 Person kein Kind</v>
+      </c>
+      <c r="G12" t="str">
+        <v>Bachelor</v>
+      </c>
+      <c r="H12" t="str">
+        <v>Schweiz</v>
+      </c>
+      <c r="I12" t="str">
+        <v>9000</v>
+      </c>
+      <c r="J12" t="str" xml:space="preserve">
+        <v xml:space="preserve">Jobbezeichnung: Digital Manager
+Jobbeschreibung: Steuert digitale Kanäle und Massnahmen, um Marken sichtbar zu machen und die Online-Performance zu steigern. Verantwortet Strategie und Umsetzung von SEO, SEA, E-Mail, Display und Social Ads. Analysiert Performance-Daten und optimiert Budgets entlang des Funnels.
+Berufserfahrung: 2-4 Jahre
+Branchenwissen: Social Media Marketing / Content Creation, Digital Marketing / Kommunikation, Social Media / Partnerschaften
+Tools &amp; Technologien: Microsoft Office / Adobe Creative Suite, Microsoft PowerPoint / Social Media Platforms (FB/TikTok/IG), Microsoft Word / CMS / Typo3
+Soziale Kompetenz: Teamwork / Teamwork / Collaboration, Leadership / Structured working style, Communication / Proactive / autonomous
+Weitere Kenntnisse: Social Media / Social Media Strategy, Sales / Content Strategy &amp; Planning, Project Management / Video &amp; Photo Production</v>
+      </c>
+    </row>
+    <row r="13" xml:space="preserve">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13" t="str">
+        <v>DMM (Digital Manager)</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Weiblich</v>
+      </c>
+      <c r="D13" t="str">
+        <v>20-29 Jahre</v>
+      </c>
+      <c r="E13" t="str">
+        <v>Schweiz</v>
+      </c>
+      <c r="F13" t="str">
+        <v>2 Personen 1 Kind</v>
+      </c>
+      <c r="G13" t="str">
+        <v>Bachelor</v>
+      </c>
+      <c r="H13" t="str">
+        <v>Schweiz</v>
+      </c>
+      <c r="I13" t="str">
+        <v>9000</v>
+      </c>
+      <c r="J13" t="str" xml:space="preserve">
+        <v xml:space="preserve">Jobbezeichnung: Digital Manager
+Jobbeschreibung: Steuert digitale Kanäle und Massnahmen, um Marken sichtbar zu machen und die Online-Performance zu steigern. Verantwortet Strategie und Umsetzung von SEO, SEA, E-Mail, Display und Social Ads. Analysiert Performance-Daten und optimiert Budgets entlang des Funnels.
+Berufserfahrung: 2-4 Jahre
+Branchenwissen: Social Media Marketing / Content Creation, Digital Marketing / Kommunikation, Social Media / Partnerschaften
+Tools &amp; Technologien: Microsoft Office / Adobe Creative Suite, Microsoft PowerPoint / Social Media Platforms (FB/TikTok/IG), Microsoft Word / CMS / Typo3
+Soziale Kompetenz: Teamwork / Teamwork / Collaboration, Leadership / Structured working style, Communication / Proactive / autonomous
+Weitere Kenntnisse: Social Media / Social Media Strategy, Sales / Content Strategy &amp; Planning, Project Management / Video &amp; Photo Production</v>
+      </c>
+    </row>
+    <row r="14" xml:space="preserve">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14" t="str">
         <v>Growth Manager</v>
       </c>
-      <c r="B5" t="str">
-        <v>Treibt skalierbares Nutzer- und Umsatzwachstum durch experimentelle Massnahmen entlang des gesamten Funnels. Nutzt Daten, Hypothesen und schnelle Tests, um Akquise, Aktivierung und Retention zu verbessern. Arbeitet eng mit Produkt, Marketing und Engineering zusammen.</v>
-      </c>
-      <c r="C5" t="str">
-        <v>Hypothesengetrieben, experimentierfreudig, analytisch, technisch versiert, ergebnisfokussiert.</v>
-      </c>
-      <c r="D5" t="str">
-        <v>Mixpanel, Amplitude, GrowthBook, A/B-Testing, SQL, North-Star-Metriken, Lean-Experimente.</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>Kommunikationsmanager</v>
-      </c>
-      <c r="B6" t="str">
-        <v>Verantwortet die interne und externe Kommunikation und sichert eine konsistente Markenstimme. Plant Pressemitteilungen, Statements, Krisenkommunikation und Stakeholder-Dialoge. Schreibt Inhalte, briefed Agenturen und steuert den Content-Kalender.</v>
-      </c>
-      <c r="C6" t="str">
-        <v>Sprachgewandt, strategisch, vertrauenswürdig, gut vernetzt, krisensicher.</v>
-      </c>
-      <c r="D6" t="str">
-        <v>PR-Tools, Newsroom-Plattformen, LinkedIn, klassische Medien, redaktionelle Workflows, Storytelling.</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>Website Manager</v>
-      </c>
-      <c r="B7" t="str">
-        <v>Verantwortet Konzeption, Pflege und Weiterentwicklung der Unternehmenswebsite. Überwacht Performance, SEO, UX und Conversion und steuert Anpassungen mit Entwicklung und Design. Sorgt für rechtssichere, barrierearme Inhalte und einen reibungslosen technischen Betrieb.</v>
-      </c>
-      <c r="C7" t="str">
-        <v>Detailgenau, technisch versiert, UX-affin, strukturiert, datengetrieben.</v>
-      </c>
-      <c r="D7" t="str">
-        <v>CMS (WordPress, Webflow, TYPO3), GA4, Search Console, Lighthouse, A/B-Testing, Figma.</v>
+      <c r="C14" t="str">
+        <v>Männlich</v>
+      </c>
+      <c r="D14" t="str">
+        <v>20-29 Jahre</v>
+      </c>
+      <c r="E14" t="str">
+        <v>Schweiz</v>
+      </c>
+      <c r="F14" t="str">
+        <v>1 Person kein Kind</v>
+      </c>
+      <c r="G14" t="str">
+        <v>Bachelor</v>
+      </c>
+      <c r="H14" t="str">
+        <v>Schweiz</v>
+      </c>
+      <c r="I14" t="str">
+        <v>9000</v>
+      </c>
+      <c r="J14" t="str" xml:space="preserve">
+        <v xml:space="preserve">Jobbezeichnung: Growth Manager
+Jobbeschreibung: Treibt skalierbares Nutzer- und Umsatzwachstum durch experimentelle Massnahmen entlang des gesamten Funnels. Nutzt Daten, Hypothesen und schnelle Tests, um Akquise, Aktivierung und Retention zu verbessern. Arbeitet eng mit Produkt, Marketing und Engineering zusammen.
+Berufserfahrung: 2-4 Jahre
+Branchenwissen: Digital Marketing / Website Development, SEO / Digital Marketing, Web Design / Website security
+Tools &amp; Technologien: WordPress / CMS (WordPress/Typo3/other), HTML / HTML / CSS, Google Analytics / Dev tools (Git/Docker/CI/CD)
+Soziale Kompetenz: Teamwork / Teamwork / Collaboration, Communication / Technical leadership, Project Management / Cross-functional collaboration
+Weitere Kenntnisse: Social Media / Technical Architecture / DevOps, SEO / Website Operations / Content Publishing, Marketing Strategy / Customer Journey / UX</v>
+      </c>
+    </row>
+    <row r="15" xml:space="preserve">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Growth Manager</v>
+      </c>
+      <c r="C15" t="str">
+        <v>Männlich</v>
+      </c>
+      <c r="D15" t="str">
+        <v>20-29 Jahre</v>
+      </c>
+      <c r="E15" t="str">
+        <v>Schweiz</v>
+      </c>
+      <c r="F15" t="str">
+        <v>2 Personen 1 Kind</v>
+      </c>
+      <c r="G15" t="str">
+        <v>Bachelor</v>
+      </c>
+      <c r="H15" t="str">
+        <v>Schweiz</v>
+      </c>
+      <c r="I15" t="str">
+        <v>9000</v>
+      </c>
+      <c r="J15" t="str" xml:space="preserve">
+        <v xml:space="preserve">Jobbezeichnung: Growth Manager
+Jobbeschreibung: Treibt skalierbares Nutzer- und Umsatzwachstum durch experimentelle Massnahmen entlang des gesamten Funnels. Nutzt Daten, Hypothesen und schnelle Tests, um Akquise, Aktivierung und Retention zu verbessern. Arbeitet eng mit Produkt, Marketing und Engineering zusammen.
+Berufserfahrung: 2-4 Jahre
+Branchenwissen: Digital Marketing / Website Development, SEO / Digital Marketing, Web Design / Website security
+Tools &amp; Technologien: WordPress / CMS (WordPress/Typo3/other), HTML / HTML / CSS, Google Analytics / Dev tools (Git/Docker/CI/CD)
+Soziale Kompetenz: Teamwork / Teamwork / Collaboration, Communication / Technical leadership, Project Management / Cross-functional collaboration
+Weitere Kenntnisse: Social Media / Technical Architecture / DevOps, SEO / Website Operations / Content Publishing, Marketing Strategy / Customer Journey / UX</v>
+      </c>
+    </row>
+    <row r="16" xml:space="preserve">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Growth Manager</v>
+      </c>
+      <c r="C16" t="str">
+        <v>Weiblich</v>
+      </c>
+      <c r="D16" t="str">
+        <v>20-29 Jahre</v>
+      </c>
+      <c r="E16" t="str">
+        <v>Schweiz</v>
+      </c>
+      <c r="F16" t="str">
+        <v>1 Person kein Kind</v>
+      </c>
+      <c r="G16" t="str">
+        <v>Bachelor</v>
+      </c>
+      <c r="H16" t="str">
+        <v>Schweiz</v>
+      </c>
+      <c r="I16" t="str">
+        <v>9000</v>
+      </c>
+      <c r="J16" t="str" xml:space="preserve">
+        <v xml:space="preserve">Jobbezeichnung: Growth Manager
+Jobbeschreibung: Treibt skalierbares Nutzer- und Umsatzwachstum durch experimentelle Massnahmen entlang des gesamten Funnels. Nutzt Daten, Hypothesen und schnelle Tests, um Akquise, Aktivierung und Retention zu verbessern. Arbeitet eng mit Produkt, Marketing und Engineering zusammen.
+Berufserfahrung: 2-4 Jahre
+Branchenwissen: Digital Marketing / Website Development, SEO / Digital Marketing, Web Design / Website security
+Tools &amp; Technologien: WordPress / CMS (WordPress/Typo3/other), HTML / HTML / CSS, Google Analytics / Dev tools (Git/Docker/CI/CD)
+Soziale Kompetenz: Teamwork / Teamwork / Collaboration, Communication / Technical leadership, Project Management / Cross-functional collaboration
+Weitere Kenntnisse: Social Media / Technical Architecture / DevOps, SEO / Website Operations / Content Publishing, Marketing Strategy / Customer Journey / UX</v>
+      </c>
+    </row>
+    <row r="17" xml:space="preserve">
+      <c r="A17">
+        <v>16</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Growth Manager</v>
+      </c>
+      <c r="C17" t="str">
+        <v>Weiblich</v>
+      </c>
+      <c r="D17" t="str">
+        <v>20-29 Jahre</v>
+      </c>
+      <c r="E17" t="str">
+        <v>Schweiz</v>
+      </c>
+      <c r="F17" t="str">
+        <v>2 Personen 1 Kind</v>
+      </c>
+      <c r="G17" t="str">
+        <v>Bachelor</v>
+      </c>
+      <c r="H17" t="str">
+        <v>Schweiz</v>
+      </c>
+      <c r="I17" t="str">
+        <v>9000</v>
+      </c>
+      <c r="J17" t="str" xml:space="preserve">
+        <v xml:space="preserve">Jobbezeichnung: Growth Manager
+Jobbeschreibung: Treibt skalierbares Nutzer- und Umsatzwachstum durch experimentelle Massnahmen entlang des gesamten Funnels. Nutzt Daten, Hypothesen und schnelle Tests, um Akquise, Aktivierung und Retention zu verbessern. Arbeitet eng mit Produkt, Marketing und Engineering zusammen.
+Berufserfahrung: 2-4 Jahre
+Branchenwissen: Digital Marketing / Website Development, SEO / Digital Marketing, Web Design / Website security
+Tools &amp; Technologien: WordPress / CMS (WordPress/Typo3/other), HTML / HTML / CSS, Google Analytics / Dev tools (Git/Docker/CI/CD)
+Soziale Kompetenz: Teamwork / Teamwork / Collaboration, Communication / Technical leadership, Project Management / Cross-functional collaboration
+Weitere Kenntnisse: Social Media / Technical Architecture / DevOps, SEO / Website Operations / Content Publishing, Marketing Strategy / Customer Journey / UX</v>
+      </c>
+    </row>
+    <row r="18" xml:space="preserve">
+      <c r="A18">
+        <v>17</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Kommunikation Manager</v>
+      </c>
+      <c r="C18" t="str">
+        <v>Männlich</v>
+      </c>
+      <c r="D18" t="str">
+        <v>20-29 Jahre</v>
+      </c>
+      <c r="E18" t="str">
+        <v>Schweiz</v>
+      </c>
+      <c r="F18" t="str">
+        <v>1 Person kein Kind</v>
+      </c>
+      <c r="G18" t="str">
+        <v>Bachelor</v>
+      </c>
+      <c r="H18" t="str">
+        <v>Schweiz</v>
+      </c>
+      <c r="I18" t="str">
+        <v>9000</v>
+      </c>
+      <c r="J18" t="str" xml:space="preserve">
+        <v xml:space="preserve">Jobbezeichnung: Kommunikationsmanager
+Jobbeschreibung: Verantwortet die interne und externe Kommunikation und sichert eine konsistente Markenstimme. Plant Pressemitteilungen, Statements, Krisenkommunikation und Stakeholder-Dialoge. Schreibt Inhalte, briefed Agenturen und steuert den Content-Kalender.
+Berufserfahrung: 4-6 Jahre
+Branchenwissen: Event Management / Kommunikation, Digital Marketing / Strategische Kommunikationsplanung, Corporate Communications / Stakeholderkommunikation
+Tools &amp; Technologien: Microsoft Office / MS 365 / Content Management Systems, Adobe InDesign / Social Media / Monitoring tools, Adobe Photoshop / Digitale Kanäle / Content Formate
+Soziale Kompetenz: Teamwork / Communication, Social Media / Teamwork / Collaboration, Communication / Strategic thinking
+Weitere Kenntnisse: Project Management / Strategic Communications, Marketing Strategy / Project Management, SEO / Leadership</v>
+      </c>
+    </row>
+    <row r="19" xml:space="preserve">
+      <c r="A19">
+        <v>18</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Kommunikation Manager</v>
+      </c>
+      <c r="C19" t="str">
+        <v>Männlich</v>
+      </c>
+      <c r="D19" t="str">
+        <v>20-29 Jahre</v>
+      </c>
+      <c r="E19" t="str">
+        <v>Schweiz</v>
+      </c>
+      <c r="F19" t="str">
+        <v>2 Personen 1 Kind</v>
+      </c>
+      <c r="G19" t="str">
+        <v>Bachelor</v>
+      </c>
+      <c r="H19" t="str">
+        <v>Schweiz</v>
+      </c>
+      <c r="I19" t="str">
+        <v>9000</v>
+      </c>
+      <c r="J19" t="str" xml:space="preserve">
+        <v xml:space="preserve">Jobbezeichnung: Kommunikationsmanager
+Jobbeschreibung: Verantwortet die interne und externe Kommunikation und sichert eine konsistente Markenstimme. Plant Pressemitteilungen, Statements, Krisenkommunikation und Stakeholder-Dialoge. Schreibt Inhalte, briefed Agenturen und steuert den Content-Kalender.
+Berufserfahrung: 4-6 Jahre
+Branchenwissen: Event Management / Kommunikation, Digital Marketing / Strategische Kommunikationsplanung, Corporate Communications / Stakeholderkommunikation
+Tools &amp; Technologien: Microsoft Office / MS 365 / Content Management Systems, Adobe InDesign / Social Media / Monitoring tools, Adobe Photoshop / Digitale Kanäle / Content Formate
+Soziale Kompetenz: Teamwork / Communication, Social Media / Teamwork / Collaboration, Communication / Strategic thinking
+Weitere Kenntnisse: Project Management / Strategic Communications, Marketing Strategy / Project Management, SEO / Leadership</v>
+      </c>
+    </row>
+    <row r="20" xml:space="preserve">
+      <c r="A20">
+        <v>19</v>
+      </c>
+      <c r="B20" t="str">
+        <v>Kommunikation Manager</v>
+      </c>
+      <c r="C20" t="str">
+        <v>Weiblich</v>
+      </c>
+      <c r="D20" t="str">
+        <v>20-29 Jahre</v>
+      </c>
+      <c r="E20" t="str">
+        <v>Schweiz</v>
+      </c>
+      <c r="F20" t="str">
+        <v>1 Person kein Kind</v>
+      </c>
+      <c r="G20" t="str">
+        <v>Bachelor</v>
+      </c>
+      <c r="H20" t="str">
+        <v>Schweiz</v>
+      </c>
+      <c r="I20" t="str">
+        <v>9000</v>
+      </c>
+      <c r="J20" t="str" xml:space="preserve">
+        <v xml:space="preserve">Jobbezeichnung: Kommunikationsmanager
+Jobbeschreibung: Verantwortet die interne und externe Kommunikation und sichert eine konsistente Markenstimme. Plant Pressemitteilungen, Statements, Krisenkommunikation und Stakeholder-Dialoge. Schreibt Inhalte, briefed Agenturen und steuert den Content-Kalender.
+Berufserfahrung: 4-6 Jahre
+Branchenwissen: Event Management / Kommunikation, Digital Marketing / Strategische Kommunikationsplanung, Corporate Communications / Stakeholderkommunikation
+Tools &amp; Technologien: Microsoft Office / MS 365 / Content Management Systems, Adobe InDesign / Social Media / Monitoring tools, Adobe Photoshop / Digitale Kanäle / Content Formate
+Soziale Kompetenz: Teamwork / Communication, Social Media / Teamwork / Collaboration, Communication / Strategic thinking
+Weitere Kenntnisse: Project Management / Strategic Communications, Marketing Strategy / Project Management, SEO / Leadership</v>
+      </c>
+    </row>
+    <row r="21" xml:space="preserve">
+      <c r="A21">
+        <v>20</v>
+      </c>
+      <c r="B21" t="str">
+        <v>Kommunikation Manager</v>
+      </c>
+      <c r="C21" t="str">
+        <v>Weiblich</v>
+      </c>
+      <c r="D21" t="str">
+        <v>20-29 Jahre</v>
+      </c>
+      <c r="E21" t="str">
+        <v>Schweiz</v>
+      </c>
+      <c r="F21" t="str">
+        <v>2 Personen 1 Kind</v>
+      </c>
+      <c r="G21" t="str">
+        <v>Bachelor</v>
+      </c>
+      <c r="H21" t="str">
+        <v>Schweiz</v>
+      </c>
+      <c r="I21" t="str">
+        <v>9000</v>
+      </c>
+      <c r="J21" t="str" xml:space="preserve">
+        <v xml:space="preserve">Jobbezeichnung: Kommunikationsmanager
+Jobbeschreibung: Verantwortet die interne und externe Kommunikation und sichert eine konsistente Markenstimme. Plant Pressemitteilungen, Statements, Krisenkommunikation und Stakeholder-Dialoge. Schreibt Inhalte, briefed Agenturen und steuert den Content-Kalender.
+Berufserfahrung: 4-6 Jahre
+Branchenwissen: Event Management / Kommunikation, Digital Marketing / Strategische Kommunikationsplanung, Corporate Communications / Stakeholderkommunikation
+Tools &amp; Technologien: Microsoft Office / MS 365 / Content Management Systems, Adobe InDesign / Social Media / Monitoring tools, Adobe Photoshop / Digitale Kanäle / Content Formate
+Soziale Kompetenz: Teamwork / Communication, Social Media / Teamwork / Collaboration, Communication / Strategic thinking
+Weitere Kenntnisse: Project Management / Strategic Communications, Marketing Strategy / Project Management, SEO / Leadership</v>
+      </c>
+    </row>
+    <row r="22" xml:space="preserve">
+      <c r="A22">
+        <v>21</v>
+      </c>
+      <c r="B22" t="str">
+        <v>Webseiten Manager</v>
+      </c>
+      <c r="C22" t="str">
+        <v>Männlich</v>
+      </c>
+      <c r="D22" t="str">
+        <v>20-29 Jahre</v>
+      </c>
+      <c r="E22" t="str">
+        <v>Schweiz</v>
+      </c>
+      <c r="F22" t="str">
+        <v>1 Person kein Kind</v>
+      </c>
+      <c r="G22" t="str">
+        <v>Bachelor</v>
+      </c>
+      <c r="H22" t="str">
+        <v>Schweiz</v>
+      </c>
+      <c r="I22" t="str">
+        <v>9000</v>
+      </c>
+      <c r="J22" t="str" xml:space="preserve">
+        <v xml:space="preserve">Jobbezeichnung: Website Manager
+Jobbeschreibung: Verantwortet Konzeption, Pflege und Weiterentwicklung der Unternehmenswebsite. Überwacht Performance, SEO, UX und Conversion und steuert Anpassungen mit Entwicklung und Design. Sorgt für rechtssichere, barrierearme Inhalte und einen reibungslosen technischen Betrieb.
+Berufserfahrung: 5-7 Jahre
+Branchenwissen: Marketing / Digital Media and publishing, Customer Service / Fintec, Blockchain, stablecoin, FMCG / AI Governance and Compliance
+Tools &amp; Technologien: Microsoft Office / Google Analytics / GA4, Microsoft Excel / Meta Ads / Google Ads, Microsoft PowerPoint / Marketing Automation platforms
+Soziale Kompetenz: Leadership / Data-driven mindset, Teamwork / Strategic thinking, Communication / Cross-functional collaboration
+Weitere Kenntnisse: Project Management / Funnel Optimization / A/B Testing, Marketing Strategy / Campaign Management, Campaign Management / Performance Marketing</v>
+      </c>
+    </row>
+    <row r="23" xml:space="preserve">
+      <c r="A23">
+        <v>22</v>
+      </c>
+      <c r="B23" t="str">
+        <v>Webseiten Manager</v>
+      </c>
+      <c r="C23" t="str">
+        <v>Männlich</v>
+      </c>
+      <c r="D23" t="str">
+        <v>20-29 Jahre</v>
+      </c>
+      <c r="E23" t="str">
+        <v>Schweiz</v>
+      </c>
+      <c r="F23" t="str">
+        <v>2 Personen 1 Kind</v>
+      </c>
+      <c r="G23" t="str">
+        <v>Bachelor</v>
+      </c>
+      <c r="H23" t="str">
+        <v>Schweiz</v>
+      </c>
+      <c r="I23" t="str">
+        <v>9000</v>
+      </c>
+      <c r="J23" t="str" xml:space="preserve">
+        <v xml:space="preserve">Jobbezeichnung: Website Manager
+Jobbeschreibung: Verantwortet Konzeption, Pflege und Weiterentwicklung der Unternehmenswebsite. Überwacht Performance, SEO, UX und Conversion und steuert Anpassungen mit Entwicklung und Design. Sorgt für rechtssichere, barrierearme Inhalte und einen reibungslosen technischen Betrieb.
+Berufserfahrung: 5-7 Jahre
+Branchenwissen: Marketing / Digital Media and publishing, Customer Service / Fintec, Blockchain, stablecoin, FMCG / AI Governance and Compliance
+Tools &amp; Technologien: Microsoft Office / Google Analytics / GA4, Microsoft Excel / Meta Ads / Google Ads, Microsoft PowerPoint / Marketing Automation platforms
+Soziale Kompetenz: Leadership / Data-driven mindset, Teamwork / Strategic thinking, Communication / Cross-functional collaboration
+Weitere Kenntnisse: Project Management / Funnel Optimization / A/B Testing, Marketing Strategy / Campaign Management, Campaign Management / Performance Marketing</v>
+      </c>
+    </row>
+    <row r="24" xml:space="preserve">
+      <c r="A24">
+        <v>23</v>
+      </c>
+      <c r="B24" t="str">
+        <v>Webseiten Manager</v>
+      </c>
+      <c r="C24" t="str">
+        <v>Weiblich</v>
+      </c>
+      <c r="D24" t="str">
+        <v>20-29 Jahre</v>
+      </c>
+      <c r="E24" t="str">
+        <v>Schweiz</v>
+      </c>
+      <c r="F24" t="str">
+        <v>1 Person kein Kind</v>
+      </c>
+      <c r="G24" t="str">
+        <v>Bachelor</v>
+      </c>
+      <c r="H24" t="str">
+        <v>Schweiz</v>
+      </c>
+      <c r="I24" t="str">
+        <v>9000</v>
+      </c>
+      <c r="J24" t="str" xml:space="preserve">
+        <v xml:space="preserve">Jobbezeichnung: Website Manager
+Jobbeschreibung: Verantwortet Konzeption, Pflege und Weiterentwicklung der Unternehmenswebsite. Überwacht Performance, SEO, UX und Conversion und steuert Anpassungen mit Entwicklung und Design. Sorgt für rechtssichere, barrierearme Inhalte und einen reibungslosen technischen Betrieb.
+Berufserfahrung: 5-7 Jahre
+Branchenwissen: Marketing / Digital Media and publishing, Customer Service / Fintec, Blockchain, stablecoin, FMCG / AI Governance and Compliance
+Tools &amp; Technologien: Microsoft Office / Google Analytics / GA4, Microsoft Excel / Meta Ads / Google Ads, Microsoft PowerPoint / Marketing Automation platforms
+Soziale Kompetenz: Leadership / Data-driven mindset, Teamwork / Strategic thinking, Communication / Cross-functional collaboration
+Weitere Kenntnisse: Project Management / Funnel Optimization / A/B Testing, Marketing Strategy / Campaign Management, Campaign Management / Performance Marketing</v>
+      </c>
+    </row>
+    <row r="25" xml:space="preserve">
+      <c r="A25">
+        <v>24</v>
+      </c>
+      <c r="B25" t="str">
+        <v>Webseiten Manager</v>
+      </c>
+      <c r="C25" t="str">
+        <v>Weiblich</v>
+      </c>
+      <c r="D25" t="str">
+        <v>20-29 Jahre</v>
+      </c>
+      <c r="E25" t="str">
+        <v>Schweiz</v>
+      </c>
+      <c r="F25" t="str">
+        <v>2 Personen 1 Kind</v>
+      </c>
+      <c r="G25" t="str">
+        <v>Bachelor</v>
+      </c>
+      <c r="H25" t="str">
+        <v>Schweiz</v>
+      </c>
+      <c r="I25" t="str">
+        <v>9000</v>
+      </c>
+      <c r="J25" t="str" xml:space="preserve">
+        <v xml:space="preserve">Jobbezeichnung: Website Manager
+Jobbeschreibung: Verantwortet Konzeption, Pflege und Weiterentwicklung der Unternehmenswebsite. Überwacht Performance, SEO, UX und Conversion und steuert Anpassungen mit Entwicklung und Design. Sorgt für rechtssichere, barrierearme Inhalte und einen reibungslosen technischen Betrieb.
+Berufserfahrung: 5-7 Jahre
+Branchenwissen: Marketing / Digital Media and publishing, Customer Service / Fintec, Blockchain, stablecoin, FMCG / AI Governance and Compliance
+Tools &amp; Technologien: Microsoft Office / Google Analytics / GA4, Microsoft Excel / Meta Ads / Google Ads, Microsoft PowerPoint / Marketing Automation platforms
+Soziale Kompetenz: Leadership / Data-driven mindset, Teamwork / Strategic thinking, Communication / Cross-functional collaboration
+Weitere Kenntnisse: Project Management / Funnel Optimization / A/B Testing, Marketing Strategy / Campaign Management, Campaign Management / Performance Marketing</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J25"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update Alter to 30-39 and adjust Berufserfahrung ranges
Code (page.tsx) und Generator-Skript verwenden jetzt Alter 30-39 Jahre und
Berufserfahrung SMM 3-5, DMM 3-4, Growth 3-4 Jahre. CEM, Kommunikation
und Webseiten unveraendert. Excel wurde neu generiert.
</commit_message>
<xml_diff>
--- a/personas_24.xlsx
+++ b/personas_24.xlsx
@@ -454,7 +454,7 @@
         <v>Männlich</v>
       </c>
       <c r="D2" t="str">
-        <v>20-29 Jahre</v>
+        <v>30-39 Jahre</v>
       </c>
       <c r="E2" t="str">
         <v>Schweiz</v>
@@ -492,7 +492,7 @@
         <v>Männlich</v>
       </c>
       <c r="D3" t="str">
-        <v>20-29 Jahre</v>
+        <v>30-39 Jahre</v>
       </c>
       <c r="E3" t="str">
         <v>Schweiz</v>
@@ -530,7 +530,7 @@
         <v>Weiblich</v>
       </c>
       <c r="D4" t="str">
-        <v>20-29 Jahre</v>
+        <v>30-39 Jahre</v>
       </c>
       <c r="E4" t="str">
         <v>Schweiz</v>
@@ -568,7 +568,7 @@
         <v>Weiblich</v>
       </c>
       <c r="D5" t="str">
-        <v>20-29 Jahre</v>
+        <v>30-39 Jahre</v>
       </c>
       <c r="E5" t="str">
         <v>Schweiz</v>
@@ -606,7 +606,7 @@
         <v>Männlich</v>
       </c>
       <c r="D6" t="str">
-        <v>20-29 Jahre</v>
+        <v>30-39 Jahre</v>
       </c>
       <c r="E6" t="str">
         <v>Schweiz</v>
@@ -626,7 +626,7 @@
       <c r="J6" t="str" xml:space="preserve">
         <v xml:space="preserve">Jobbezeichnung: Social Media Manager
 Jobbeschreibung: Plant, erstellt und veröffentlicht Inhalte auf Social-Media-Kanälen und steuert das Community-Management. Beobachtet Trends, KPIs und Reichweiten, um Content-Strategien laufend zu optimieren. Setzt Paid- und Organic-Kampagnen zur Markenstärkung und Lead-Generierung um.
-Berufserfahrung: 2-5 Jahre
+Berufserfahrung: 3-5 Jahre
 Branchenwissen: Digital Marketing, Marketing, E-Commerce
 Tools &amp; Technologien: Microsoft Office / Analytics &amp; BI (Tableau/Looker/Power BI), Google Analytics / CMS (WordPress/Typo3/other), Microsoft Excel / Google Ads / Google Marketing Suite
 Soziale Kompetenz: Teamwork / Teamwork / Collaboration, Communication / Analytical thinking, Project Management / Proactive / autonomous working style
@@ -644,7 +644,7 @@
         <v>Männlich</v>
       </c>
       <c r="D7" t="str">
-        <v>20-29 Jahre</v>
+        <v>30-39 Jahre</v>
       </c>
       <c r="E7" t="str">
         <v>Schweiz</v>
@@ -664,7 +664,7 @@
       <c r="J7" t="str" xml:space="preserve">
         <v xml:space="preserve">Jobbezeichnung: Social Media Manager
 Jobbeschreibung: Plant, erstellt und veröffentlicht Inhalte auf Social-Media-Kanälen und steuert das Community-Management. Beobachtet Trends, KPIs und Reichweiten, um Content-Strategien laufend zu optimieren. Setzt Paid- und Organic-Kampagnen zur Markenstärkung und Lead-Generierung um.
-Berufserfahrung: 2-5 Jahre
+Berufserfahrung: 3-5 Jahre
 Branchenwissen: Digital Marketing, Marketing, E-Commerce
 Tools &amp; Technologien: Microsoft Office / Analytics &amp; BI (Tableau/Looker/Power BI), Google Analytics / CMS (WordPress/Typo3/other), Microsoft Excel / Google Ads / Google Marketing Suite
 Soziale Kompetenz: Teamwork / Teamwork / Collaboration, Communication / Analytical thinking, Project Management / Proactive / autonomous working style
@@ -682,7 +682,7 @@
         <v>Weiblich</v>
       </c>
       <c r="D8" t="str">
-        <v>20-29 Jahre</v>
+        <v>30-39 Jahre</v>
       </c>
       <c r="E8" t="str">
         <v>Schweiz</v>
@@ -702,7 +702,7 @@
       <c r="J8" t="str" xml:space="preserve">
         <v xml:space="preserve">Jobbezeichnung: Social Media Manager
 Jobbeschreibung: Plant, erstellt und veröffentlicht Inhalte auf Social-Media-Kanälen und steuert das Community-Management. Beobachtet Trends, KPIs und Reichweiten, um Content-Strategien laufend zu optimieren. Setzt Paid- und Organic-Kampagnen zur Markenstärkung und Lead-Generierung um.
-Berufserfahrung: 2-5 Jahre
+Berufserfahrung: 3-5 Jahre
 Branchenwissen: Digital Marketing, Marketing, E-Commerce
 Tools &amp; Technologien: Microsoft Office / Analytics &amp; BI (Tableau/Looker/Power BI), Google Analytics / CMS (WordPress/Typo3/other), Microsoft Excel / Google Ads / Google Marketing Suite
 Soziale Kompetenz: Teamwork / Teamwork / Collaboration, Communication / Analytical thinking, Project Management / Proactive / autonomous working style
@@ -720,7 +720,7 @@
         <v>Weiblich</v>
       </c>
       <c r="D9" t="str">
-        <v>20-29 Jahre</v>
+        <v>30-39 Jahre</v>
       </c>
       <c r="E9" t="str">
         <v>Schweiz</v>
@@ -740,7 +740,7 @@
       <c r="J9" t="str" xml:space="preserve">
         <v xml:space="preserve">Jobbezeichnung: Social Media Manager
 Jobbeschreibung: Plant, erstellt und veröffentlicht Inhalte auf Social-Media-Kanälen und steuert das Community-Management. Beobachtet Trends, KPIs und Reichweiten, um Content-Strategien laufend zu optimieren. Setzt Paid- und Organic-Kampagnen zur Markenstärkung und Lead-Generierung um.
-Berufserfahrung: 2-5 Jahre
+Berufserfahrung: 3-5 Jahre
 Branchenwissen: Digital Marketing, Marketing, E-Commerce
 Tools &amp; Technologien: Microsoft Office / Analytics &amp; BI (Tableau/Looker/Power BI), Google Analytics / CMS (WordPress/Typo3/other), Microsoft Excel / Google Ads / Google Marketing Suite
 Soziale Kompetenz: Teamwork / Teamwork / Collaboration, Communication / Analytical thinking, Project Management / Proactive / autonomous working style
@@ -758,7 +758,7 @@
         <v>Männlich</v>
       </c>
       <c r="D10" t="str">
-        <v>20-29 Jahre</v>
+        <v>30-39 Jahre</v>
       </c>
       <c r="E10" t="str">
         <v>Schweiz</v>
@@ -778,7 +778,7 @@
       <c r="J10" t="str" xml:space="preserve">
         <v xml:space="preserve">Jobbezeichnung: Digital Manager
 Jobbeschreibung: Steuert digitale Kanäle und Massnahmen, um Marken sichtbar zu machen und die Online-Performance zu steigern. Verantwortet Strategie und Umsetzung von SEO, SEA, E-Mail, Display und Social Ads. Analysiert Performance-Daten und optimiert Budgets entlang des Funnels.
-Berufserfahrung: 2-4 Jahre
+Berufserfahrung: 3-4 Jahre
 Branchenwissen: Social Media Marketing / Content Creation, Digital Marketing / Kommunikation, Social Media / Partnerschaften
 Tools &amp; Technologien: Microsoft Office / Adobe Creative Suite, Microsoft PowerPoint / Social Media Platforms (FB/TikTok/IG), Microsoft Word / CMS / Typo3
 Soziale Kompetenz: Teamwork / Teamwork / Collaboration, Leadership / Structured working style, Communication / Proactive / autonomous
@@ -796,7 +796,7 @@
         <v>Männlich</v>
       </c>
       <c r="D11" t="str">
-        <v>20-29 Jahre</v>
+        <v>30-39 Jahre</v>
       </c>
       <c r="E11" t="str">
         <v>Schweiz</v>
@@ -816,7 +816,7 @@
       <c r="J11" t="str" xml:space="preserve">
         <v xml:space="preserve">Jobbezeichnung: Digital Manager
 Jobbeschreibung: Steuert digitale Kanäle und Massnahmen, um Marken sichtbar zu machen und die Online-Performance zu steigern. Verantwortet Strategie und Umsetzung von SEO, SEA, E-Mail, Display und Social Ads. Analysiert Performance-Daten und optimiert Budgets entlang des Funnels.
-Berufserfahrung: 2-4 Jahre
+Berufserfahrung: 3-4 Jahre
 Branchenwissen: Social Media Marketing / Content Creation, Digital Marketing / Kommunikation, Social Media / Partnerschaften
 Tools &amp; Technologien: Microsoft Office / Adobe Creative Suite, Microsoft PowerPoint / Social Media Platforms (FB/TikTok/IG), Microsoft Word / CMS / Typo3
 Soziale Kompetenz: Teamwork / Teamwork / Collaboration, Leadership / Structured working style, Communication / Proactive / autonomous
@@ -834,7 +834,7 @@
         <v>Weiblich</v>
       </c>
       <c r="D12" t="str">
-        <v>20-29 Jahre</v>
+        <v>30-39 Jahre</v>
       </c>
       <c r="E12" t="str">
         <v>Schweiz</v>
@@ -854,7 +854,7 @@
       <c r="J12" t="str" xml:space="preserve">
         <v xml:space="preserve">Jobbezeichnung: Digital Manager
 Jobbeschreibung: Steuert digitale Kanäle und Massnahmen, um Marken sichtbar zu machen und die Online-Performance zu steigern. Verantwortet Strategie und Umsetzung von SEO, SEA, E-Mail, Display und Social Ads. Analysiert Performance-Daten und optimiert Budgets entlang des Funnels.
-Berufserfahrung: 2-4 Jahre
+Berufserfahrung: 3-4 Jahre
 Branchenwissen: Social Media Marketing / Content Creation, Digital Marketing / Kommunikation, Social Media / Partnerschaften
 Tools &amp; Technologien: Microsoft Office / Adobe Creative Suite, Microsoft PowerPoint / Social Media Platforms (FB/TikTok/IG), Microsoft Word / CMS / Typo3
 Soziale Kompetenz: Teamwork / Teamwork / Collaboration, Leadership / Structured working style, Communication / Proactive / autonomous
@@ -872,7 +872,7 @@
         <v>Weiblich</v>
       </c>
       <c r="D13" t="str">
-        <v>20-29 Jahre</v>
+        <v>30-39 Jahre</v>
       </c>
       <c r="E13" t="str">
         <v>Schweiz</v>
@@ -892,7 +892,7 @@
       <c r="J13" t="str" xml:space="preserve">
         <v xml:space="preserve">Jobbezeichnung: Digital Manager
 Jobbeschreibung: Steuert digitale Kanäle und Massnahmen, um Marken sichtbar zu machen und die Online-Performance zu steigern. Verantwortet Strategie und Umsetzung von SEO, SEA, E-Mail, Display und Social Ads. Analysiert Performance-Daten und optimiert Budgets entlang des Funnels.
-Berufserfahrung: 2-4 Jahre
+Berufserfahrung: 3-4 Jahre
 Branchenwissen: Social Media Marketing / Content Creation, Digital Marketing / Kommunikation, Social Media / Partnerschaften
 Tools &amp; Technologien: Microsoft Office / Adobe Creative Suite, Microsoft PowerPoint / Social Media Platforms (FB/TikTok/IG), Microsoft Word / CMS / Typo3
 Soziale Kompetenz: Teamwork / Teamwork / Collaboration, Leadership / Structured working style, Communication / Proactive / autonomous
@@ -910,7 +910,7 @@
         <v>Männlich</v>
       </c>
       <c r="D14" t="str">
-        <v>20-29 Jahre</v>
+        <v>30-39 Jahre</v>
       </c>
       <c r="E14" t="str">
         <v>Schweiz</v>
@@ -930,7 +930,7 @@
       <c r="J14" t="str" xml:space="preserve">
         <v xml:space="preserve">Jobbezeichnung: Growth Manager
 Jobbeschreibung: Treibt skalierbares Nutzer- und Umsatzwachstum durch experimentelle Massnahmen entlang des gesamten Funnels. Nutzt Daten, Hypothesen und schnelle Tests, um Akquise, Aktivierung und Retention zu verbessern. Arbeitet eng mit Produkt, Marketing und Engineering zusammen.
-Berufserfahrung: 2-4 Jahre
+Berufserfahrung: 3-4 Jahre
 Branchenwissen: Digital Marketing / Website Development, SEO / Digital Marketing, Web Design / Website security
 Tools &amp; Technologien: WordPress / CMS (WordPress/Typo3/other), HTML / HTML / CSS, Google Analytics / Dev tools (Git/Docker/CI/CD)
 Soziale Kompetenz: Teamwork / Teamwork / Collaboration, Communication / Technical leadership, Project Management / Cross-functional collaboration
@@ -948,7 +948,7 @@
         <v>Männlich</v>
       </c>
       <c r="D15" t="str">
-        <v>20-29 Jahre</v>
+        <v>30-39 Jahre</v>
       </c>
       <c r="E15" t="str">
         <v>Schweiz</v>
@@ -968,7 +968,7 @@
       <c r="J15" t="str" xml:space="preserve">
         <v xml:space="preserve">Jobbezeichnung: Growth Manager
 Jobbeschreibung: Treibt skalierbares Nutzer- und Umsatzwachstum durch experimentelle Massnahmen entlang des gesamten Funnels. Nutzt Daten, Hypothesen und schnelle Tests, um Akquise, Aktivierung und Retention zu verbessern. Arbeitet eng mit Produkt, Marketing und Engineering zusammen.
-Berufserfahrung: 2-4 Jahre
+Berufserfahrung: 3-4 Jahre
 Branchenwissen: Digital Marketing / Website Development, SEO / Digital Marketing, Web Design / Website security
 Tools &amp; Technologien: WordPress / CMS (WordPress/Typo3/other), HTML / HTML / CSS, Google Analytics / Dev tools (Git/Docker/CI/CD)
 Soziale Kompetenz: Teamwork / Teamwork / Collaboration, Communication / Technical leadership, Project Management / Cross-functional collaboration
@@ -986,7 +986,7 @@
         <v>Weiblich</v>
       </c>
       <c r="D16" t="str">
-        <v>20-29 Jahre</v>
+        <v>30-39 Jahre</v>
       </c>
       <c r="E16" t="str">
         <v>Schweiz</v>
@@ -1006,7 +1006,7 @@
       <c r="J16" t="str" xml:space="preserve">
         <v xml:space="preserve">Jobbezeichnung: Growth Manager
 Jobbeschreibung: Treibt skalierbares Nutzer- und Umsatzwachstum durch experimentelle Massnahmen entlang des gesamten Funnels. Nutzt Daten, Hypothesen und schnelle Tests, um Akquise, Aktivierung und Retention zu verbessern. Arbeitet eng mit Produkt, Marketing und Engineering zusammen.
-Berufserfahrung: 2-4 Jahre
+Berufserfahrung: 3-4 Jahre
 Branchenwissen: Digital Marketing / Website Development, SEO / Digital Marketing, Web Design / Website security
 Tools &amp; Technologien: WordPress / CMS (WordPress/Typo3/other), HTML / HTML / CSS, Google Analytics / Dev tools (Git/Docker/CI/CD)
 Soziale Kompetenz: Teamwork / Teamwork / Collaboration, Communication / Technical leadership, Project Management / Cross-functional collaboration
@@ -1024,7 +1024,7 @@
         <v>Weiblich</v>
       </c>
       <c r="D17" t="str">
-        <v>20-29 Jahre</v>
+        <v>30-39 Jahre</v>
       </c>
       <c r="E17" t="str">
         <v>Schweiz</v>
@@ -1044,7 +1044,7 @@
       <c r="J17" t="str" xml:space="preserve">
         <v xml:space="preserve">Jobbezeichnung: Growth Manager
 Jobbeschreibung: Treibt skalierbares Nutzer- und Umsatzwachstum durch experimentelle Massnahmen entlang des gesamten Funnels. Nutzt Daten, Hypothesen und schnelle Tests, um Akquise, Aktivierung und Retention zu verbessern. Arbeitet eng mit Produkt, Marketing und Engineering zusammen.
-Berufserfahrung: 2-4 Jahre
+Berufserfahrung: 3-4 Jahre
 Branchenwissen: Digital Marketing / Website Development, SEO / Digital Marketing, Web Design / Website security
 Tools &amp; Technologien: WordPress / CMS (WordPress/Typo3/other), HTML / HTML / CSS, Google Analytics / Dev tools (Git/Docker/CI/CD)
 Soziale Kompetenz: Teamwork / Teamwork / Collaboration, Communication / Technical leadership, Project Management / Cross-functional collaboration
@@ -1062,7 +1062,7 @@
         <v>Männlich</v>
       </c>
       <c r="D18" t="str">
-        <v>20-29 Jahre</v>
+        <v>30-39 Jahre</v>
       </c>
       <c r="E18" t="str">
         <v>Schweiz</v>
@@ -1100,7 +1100,7 @@
         <v>Männlich</v>
       </c>
       <c r="D19" t="str">
-        <v>20-29 Jahre</v>
+        <v>30-39 Jahre</v>
       </c>
       <c r="E19" t="str">
         <v>Schweiz</v>
@@ -1138,7 +1138,7 @@
         <v>Weiblich</v>
       </c>
       <c r="D20" t="str">
-        <v>20-29 Jahre</v>
+        <v>30-39 Jahre</v>
       </c>
       <c r="E20" t="str">
         <v>Schweiz</v>
@@ -1176,7 +1176,7 @@
         <v>Weiblich</v>
       </c>
       <c r="D21" t="str">
-        <v>20-29 Jahre</v>
+        <v>30-39 Jahre</v>
       </c>
       <c r="E21" t="str">
         <v>Schweiz</v>
@@ -1214,7 +1214,7 @@
         <v>Männlich</v>
       </c>
       <c r="D22" t="str">
-        <v>20-29 Jahre</v>
+        <v>30-39 Jahre</v>
       </c>
       <c r="E22" t="str">
         <v>Schweiz</v>
@@ -1252,7 +1252,7 @@
         <v>Männlich</v>
       </c>
       <c r="D23" t="str">
-        <v>20-29 Jahre</v>
+        <v>30-39 Jahre</v>
       </c>
       <c r="E23" t="str">
         <v>Schweiz</v>
@@ -1290,7 +1290,7 @@
         <v>Weiblich</v>
       </c>
       <c r="D24" t="str">
-        <v>20-29 Jahre</v>
+        <v>30-39 Jahre</v>
       </c>
       <c r="E24" t="str">
         <v>Schweiz</v>
@@ -1328,7 +1328,7 @@
         <v>Weiblich</v>
       </c>
       <c r="D25" t="str">
-        <v>20-29 Jahre</v>
+        <v>30-39 Jahre</v>
       </c>
       <c r="E25" t="str">
         <v>Schweiz</v>

</xml_diff>